<commit_message>
Update published master datasets (2026-03-12)
</commit_message>
<xml_diff>
--- a/archive/InnovateUK_Funding_Opportunities_Latest_2026-03-12.xlsx
+++ b/archive/InnovateUK_Funding_Opportunities_Latest_2026-03-12.xlsx
@@ -895,7 +895,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:N5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -973,26 +973,26 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Innovate Funding Service</t>
+          <t>Innovate UK Business Connect</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Clean Maritime Demonstration Competition 7: Pre-deployment trials</t>
+          <t>Clean Maritime Demonstration Competition 7</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2415/overview/fa34afe8-b2e7-4cda-b77b-cf952d26a27a</t>
+          <t>https://iuk-business-connect.org.uk/opportunities/clean-maritime-demonstration-competition-7/</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-11 10:34</t>
+          <t>2026-03-12 10:27</t>
         </is>
       </c>
       <c r="E2" s="1" t="n">
-        <v>46092.44027777778</v>
+        <v>46093.43541666667</v>
       </c>
       <c r="F2" t="b">
         <v>1</v>
@@ -1001,11 +1001,17 @@
       <c r="H2" t="b">
         <v>0</v>
       </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>11/03/2026</t>
+        </is>
+      </c>
+      <c r="J2" s="1" t="n">
+        <v>46092</v>
+      </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Wednesday 15 July 2026 11:00am</t>
+          <t>15/07/2026                              11:00</t>
         </is>
       </c>
       <c r="L2" s="1" t="n">
@@ -1013,7 +1019,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>£6.0 million</t>
+          <t>£121.0 million</t>
         </is>
       </c>
       <c r="N2" s="1" t="n">
@@ -1028,12 +1034,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Clean Maritime Demonstration Competition 7: Feasibility studies</t>
+          <t>Clean Maritime Demonstration Competition 7: Pre-deployment trials</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2416/overview/f49610a2-5e82-4898-b357-10f80154a2b8</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2415/overview/fa34afe8-b2e7-4cda-b77b-cf952d26a27a</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -1063,7 +1069,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>£1.0 million</t>
+          <t>£6.0 million</t>
         </is>
       </c>
       <c r="N3" s="1" t="n">
@@ -1078,12 +1084,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Clean Maritime Demonstration Competition 7: Deployment trials</t>
+          <t>Clean Maritime Demonstration Competition 7: Feasibility studies</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2414/overview/3409b968-a2b7-44e7-83a7-c2d3e8ad8f8e</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2416/overview/f49610a2-5e82-4898-b357-10f80154a2b8</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -1113,10 +1119,60 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
+          <t>£1.0 million</t>
+        </is>
+      </c>
+      <c r="N4" s="1" t="n">
+        <v>46092</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Innovate Funding Service</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Clean Maritime Demonstration Competition 7: Deployment trials</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2414/overview/3409b968-a2b7-44e7-83a7-c2d3e8ad8f8e</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2026-03-11 10:34</t>
+        </is>
+      </c>
+      <c r="E5" s="1" t="n">
+        <v>46092.44027777778</v>
+      </c>
+      <c r="F5" t="b">
+        <v>1</v>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="b">
+        <v>0</v>
+      </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Wednesday 15 July 2026 11:00am</t>
+        </is>
+      </c>
+      <c r="L5" s="1" t="n">
+        <v>46218.45833333334</v>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
           <t>£15.0 million</t>
         </is>
       </c>
-      <c r="N4" s="1" t="n">
+      <c r="N5" s="1" t="n">
         <v>46092</v>
       </c>
     </row>
@@ -1164,10 +1220,10 @@
         <v>3</v>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3">
@@ -1727,7 +1783,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N284"/>
+  <dimension ref="A1:N285"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10509,26 +10565,26 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>Innovate Funding Service</t>
+          <t>Innovate UK Business Connect</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>Future Leaders Fellowships: Round 10, business and non-academic</t>
+          <t>Clean Maritime Demonstration Competition 7</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2058/overview/0f904547-f415-4fb9-94a7-0701c38a2ba1</t>
+          <t>https://iuk-business-connect.org.uk/opportunities/clean-maritime-demonstration-competition-7/</t>
         </is>
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>2025-06-14 08:41</t>
+          <t>2026-03-12 10:27</t>
         </is>
       </c>
       <c r="E173" s="1" t="n">
-        <v>45822.36180555556</v>
+        <v>46093.43541666667</v>
       </c>
       <c r="F173" t="b">
         <v>1</v>
@@ -10537,23 +10593,29 @@
       <c r="H173" t="b">
         <v>0</v>
       </c>
-      <c r="I173" t="inlineStr"/>
-      <c r="J173" t="inlineStr"/>
+      <c r="I173" t="inlineStr">
+        <is>
+          <t>11/03/2026</t>
+        </is>
+      </c>
+      <c r="J173" s="1" t="n">
+        <v>46092</v>
+      </c>
       <c r="K173" t="inlineStr">
         <is>
-          <t>Wednesday 5 November 2025 11:00am</t>
+          <t>15/07/2026                              11:00</t>
         </is>
       </c>
       <c r="L173" s="1" t="n">
-        <v>45966.45833333334</v>
+        <v>46218.45833333334</v>
       </c>
       <c r="M173" t="inlineStr">
         <is>
-          <t>£3.0 million</t>
+          <t>£121.0 million</t>
         </is>
       </c>
       <c r="N173" s="1" t="n">
-        <v>45819</v>
+        <v>46092</v>
       </c>
     </row>
     <row r="174">
@@ -10564,12 +10626,12 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>ADOPT Facilitator Support Grant: Round 2</t>
+          <t>Future Leaders Fellowships: Round 10, business and non-academic</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2223/overview/4e423e05-3228-45e3-9cfe-0b39d1227307</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2058/overview/0f904547-f415-4fb9-94a7-0701c38a2ba1</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
@@ -10591,15 +10653,15 @@
       <c r="J174" t="inlineStr"/>
       <c r="K174" t="inlineStr">
         <is>
-          <t>Thursday 24 July 2025 11:00am</t>
+          <t>Wednesday 5 November 2025 11:00am</t>
         </is>
       </c>
       <c r="L174" s="1" t="n">
-        <v>45862.45833333334</v>
+        <v>45966.45833333334</v>
       </c>
       <c r="M174" t="inlineStr">
         <is>
-          <t>£2,500</t>
+          <t>£3.0 million</t>
         </is>
       </c>
       <c r="N174" s="1" t="n">
@@ -10614,12 +10676,12 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>MSI Improving energy or resource efficiency in manufacturing FS</t>
+          <t>ADOPT Facilitator Support Grant: Round 2</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2225/overview/c43ef163-3872-4178-b80d-88c406691610</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2223/overview/4e423e05-3228-45e3-9cfe-0b39d1227307</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
@@ -10641,15 +10703,15 @@
       <c r="J175" t="inlineStr"/>
       <c r="K175" t="inlineStr">
         <is>
-          <t>Wednesday 2 July 2025 11:00am</t>
+          <t>Thursday 24 July 2025 11:00am</t>
         </is>
       </c>
       <c r="L175" s="1" t="n">
-        <v>45840.45833333334</v>
+        <v>45862.45833333334</v>
       </c>
       <c r="M175" t="inlineStr">
         <is>
-          <t>£100,000</t>
+          <t>£2,500</t>
         </is>
       </c>
       <c r="N175" s="1" t="n">
@@ -10664,12 +10726,12 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>New Innovators in Marine and Maritime, Great South West</t>
+          <t>MSI Improving energy or resource efficiency in manufacturing FS</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2215/overview/67b86d6c-bab9-4a01-aacc-3da2e57edc99</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2225/overview/c43ef163-3872-4178-b80d-88c406691610</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
@@ -10699,7 +10761,7 @@
       </c>
       <c r="M176" t="inlineStr">
         <is>
-          <t>£50,000</t>
+          <t>£100,000</t>
         </is>
       </c>
       <c r="N176" s="1" t="n">
@@ -10714,12 +10776,12 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>Commercialising Knowledge Assets Fund (CKAF) Autumn</t>
+          <t>New Innovators in Marine and Maritime, Great South West</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2217/overview/c555f64e-5485-4e49-89b8-32d61fac4ff0</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2215/overview/67b86d6c-bab9-4a01-aacc-3da2e57edc99</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
@@ -10741,15 +10803,15 @@
       <c r="J177" t="inlineStr"/>
       <c r="K177" t="inlineStr">
         <is>
-          <t>Thursday 4 September 2025 11:00am</t>
+          <t>Wednesday 2 July 2025 11:00am</t>
         </is>
       </c>
       <c r="L177" s="1" t="n">
-        <v>45904.45833333334</v>
+        <v>45840.45833333334</v>
       </c>
       <c r="M177" t="inlineStr">
         <is>
-          <t>£250,000</t>
+          <t>£50,000</t>
         </is>
       </c>
       <c r="N177" s="1" t="n">
@@ -10764,12 +10826,12 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>ATI Programme strategic batch: EoI – June 2025</t>
+          <t>Commercialising Knowledge Assets Fund (CKAF) Autumn</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2218/overview/a45dcc8a-b621-4a79-9e4d-046e19b6b1e9</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2217/overview/c555f64e-5485-4e49-89b8-32d61fac4ff0</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
@@ -10791,13 +10853,17 @@
       <c r="J178" t="inlineStr"/>
       <c r="K178" t="inlineStr">
         <is>
-          <t>Wednesday 18 June 2025 11:00am</t>
+          <t>Thursday 4 September 2025 11:00am</t>
         </is>
       </c>
       <c r="L178" s="1" t="n">
-        <v>45826.45833333334</v>
-      </c>
-      <c r="M178" t="inlineStr"/>
+        <v>45904.45833333334</v>
+      </c>
+      <c r="M178" t="inlineStr">
+        <is>
+          <t>£250,000</t>
+        </is>
+      </c>
       <c r="N178" s="1" t="n">
         <v>45819</v>
       </c>
@@ -10810,12 +10876,12 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>Defra Farming Innovation Investor Partnership</t>
+          <t>ATI Programme strategic batch: EoI – June 2025</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2207/overview/05e5263b-75a1-49a0-87f0-261541af0840</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2218/overview/a45dcc8a-b621-4a79-9e4d-046e19b6b1e9</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
@@ -10837,17 +10903,13 @@
       <c r="J179" t="inlineStr"/>
       <c r="K179" t="inlineStr">
         <is>
-          <t>Wednesday 2 July 2025 11:00am</t>
+          <t>Wednesday 18 June 2025 11:00am</t>
         </is>
       </c>
       <c r="L179" s="1" t="n">
-        <v>45840.45833333334</v>
-      </c>
-      <c r="M179" t="inlineStr">
-        <is>
-          <t>£3.0 million</t>
-        </is>
-      </c>
+        <v>45826.45833333334</v>
+      </c>
+      <c r="M179" t="inlineStr"/>
       <c r="N179" s="1" t="n">
         <v>45819</v>
       </c>
@@ -10860,12 +10922,12 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>Ofgem Strategic Innovation Fund Round 5 Discovery C3</t>
+          <t>Defra Farming Innovation Investor Partnership</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2204/overview/9da241b9-1fd8-49fb-b8d0-4a81a637b3b5</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2207/overview/05e5263b-75a1-49a0-87f0-261541af0840</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
@@ -10887,15 +10949,15 @@
       <c r="J180" t="inlineStr"/>
       <c r="K180" t="inlineStr">
         <is>
-          <t>Wednesday 25 June 2025 11:00am</t>
+          <t>Wednesday 2 July 2025 11:00am</t>
         </is>
       </c>
       <c r="L180" s="1" t="n">
-        <v>45833.45833333334</v>
+        <v>45840.45833333334</v>
       </c>
       <c r="M180" t="inlineStr">
         <is>
-          <t>£150,000</t>
+          <t>£3.0 million</t>
         </is>
       </c>
       <c r="N180" s="1" t="n">
@@ -10910,12 +10972,12 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>Ofgem Strategic Innovation Fund Round 4 Discovery C3</t>
+          <t>Ofgem Strategic Innovation Fund Round 5 Discovery C3</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2200/overview/0f0721c8-5a37-4046-8e4f-7649194e8adc</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2204/overview/9da241b9-1fd8-49fb-b8d0-4a81a637b3b5</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
@@ -10960,12 +11022,12 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>Contracts for Innovation: Scaling community initiatives in diet and exercise</t>
+          <t>Ofgem Strategic Innovation Fund Round 4 Discovery C3</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2191/overview/6a097cf8-8f81-495d-b56f-3f240cfde64c</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2200/overview/0f0721c8-5a37-4046-8e4f-7649194e8adc</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
@@ -10987,15 +11049,15 @@
       <c r="J182" t="inlineStr"/>
       <c r="K182" t="inlineStr">
         <is>
-          <t>Wednesday 18 June 2025 11:00am</t>
+          <t>Wednesday 25 June 2025 11:00am</t>
         </is>
       </c>
       <c r="L182" s="1" t="n">
-        <v>45826.45833333334</v>
+        <v>45833.45833333334</v>
       </c>
       <c r="M182" t="inlineStr">
         <is>
-          <t>£250,000</t>
+          <t>£150,000</t>
         </is>
       </c>
       <c r="N182" s="1" t="n">
@@ -11010,12 +11072,12 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>Contracts for Innovation: Quantum Sensors and PNT Missions Primer</t>
+          <t>Contracts for Innovation: Scaling community initiatives in diet and exercise</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2209/overview/28f8801b-a8b3-48c8-8c81-64d75341b81d</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2191/overview/6a097cf8-8f81-495d-b56f-3f240cfde64c</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
@@ -11037,15 +11099,15 @@
       <c r="J183" t="inlineStr"/>
       <c r="K183" t="inlineStr">
         <is>
-          <t>Wednesday 2 July 2025 11:00am</t>
+          <t>Wednesday 18 June 2025 11:00am</t>
         </is>
       </c>
       <c r="L183" s="1" t="n">
-        <v>45840.45833333334</v>
+        <v>45826.45833333334</v>
       </c>
       <c r="M183" t="inlineStr">
         <is>
-          <t>£1.5 million</t>
+          <t>£250,000</t>
         </is>
       </c>
       <c r="N183" s="1" t="n">
@@ -11060,12 +11122,12 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>Contracts for Innovation: Net Zero Living Tech Trials, phase 3</t>
+          <t>Contracts for Innovation: Quantum Sensors and PNT Missions Primer</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2189/overview/a59ac38e-662b-49a5-b7f9-a44c2cc38c61</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2209/overview/28f8801b-a8b3-48c8-8c81-64d75341b81d</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
@@ -11087,15 +11149,15 @@
       <c r="J184" t="inlineStr"/>
       <c r="K184" t="inlineStr">
         <is>
-          <t>Wednesday 25 June 2025 11:00am</t>
+          <t>Wednesday 2 July 2025 11:00am</t>
         </is>
       </c>
       <c r="L184" s="1" t="n">
-        <v>45833.45833333334</v>
+        <v>45840.45833333334</v>
       </c>
       <c r="M184" t="inlineStr">
         <is>
-          <t>£100,000</t>
+          <t>£1.5 million</t>
         </is>
       </c>
       <c r="N184" s="1" t="n">
@@ -11110,12 +11172,12 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>Contracts for Innovation: Clean Air, Phase 3</t>
+          <t>Contracts for Innovation: Net Zero Living Tech Trials, phase 3</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2181/overview/02aad9d2-c984-4bd5-a3f6-80f25ec62870</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2189/overview/a59ac38e-662b-49a5-b7f9-a44c2cc38c61</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
@@ -11160,12 +11222,12 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>Contracts for Innovation: DSbD Advancing CHERI Tools and software</t>
+          <t>Contracts for Innovation: Clean Air, Phase 3</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2194/overview/91c68630-20eb-4247-8296-ae1737637756</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2181/overview/02aad9d2-c984-4bd5-a3f6-80f25ec62870</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
@@ -11187,15 +11249,15 @@
       <c r="J186" t="inlineStr"/>
       <c r="K186" t="inlineStr">
         <is>
-          <t>Wednesday 18 June 2025 11:00am</t>
+          <t>Wednesday 25 June 2025 11:00am</t>
         </is>
       </c>
       <c r="L186" s="1" t="n">
-        <v>45826.45833333334</v>
+        <v>45833.45833333334</v>
       </c>
       <c r="M186" t="inlineStr">
         <is>
-          <t>£3.0 million</t>
+          <t>£100,000</t>
         </is>
       </c>
       <c r="N186" s="1" t="n">
@@ -11210,12 +11272,12 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>Contracts for Innovation: DSbD Advancing CHERI RISC-V Devices</t>
+          <t>Contracts for Innovation: DSbD Advancing CHERI Tools and software</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2198/overview/b2e2fd41-d372-4e33-a6df-8bfefb8de0f9</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2194/overview/91c68630-20eb-4247-8296-ae1737637756</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
@@ -11245,7 +11307,7 @@
       </c>
       <c r="M187" t="inlineStr">
         <is>
-          <t>£5.0 million</t>
+          <t>£3.0 million</t>
         </is>
       </c>
       <c r="N187" s="1" t="n">
@@ -11260,12 +11322,12 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>Canada-UK Semiconductors</t>
+          <t>Contracts for Innovation: DSbD Advancing CHERI RISC-V Devices</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2192/overview/3906cbd5-fec2-4c1f-897d-ccab071708b3</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2198/overview/b2e2fd41-d372-4e33-a6df-8bfefb8de0f9</t>
         </is>
       </c>
       <c r="D188" t="inlineStr">
@@ -11287,15 +11349,15 @@
       <c r="J188" t="inlineStr"/>
       <c r="K188" t="inlineStr">
         <is>
-          <t>Wednesday 15 October 2025 11:00am</t>
+          <t>Wednesday 18 June 2025 11:00am</t>
         </is>
       </c>
       <c r="L188" s="1" t="n">
-        <v>45945.45833333334</v>
+        <v>45826.45833333334</v>
       </c>
       <c r="M188" t="inlineStr">
         <is>
-          <t>£500,000</t>
+          <t>£5.0 million</t>
         </is>
       </c>
       <c r="N188" s="1" t="n">
@@ -11310,12 +11372,12 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>Accelerated Knowledge Transfer 4 (AKT4) Addiction</t>
+          <t>Canada-UK Semiconductors</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2178/overview/2699060f-dd6f-415b-ae47-bead15aa430e</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2192/overview/3906cbd5-fec2-4c1f-897d-ccab071708b3</t>
         </is>
       </c>
       <c r="D189" t="inlineStr">
@@ -11337,15 +11399,15 @@
       <c r="J189" t="inlineStr"/>
       <c r="K189" t="inlineStr">
         <is>
-          <t>Wednesday 2 July 2025 11:00am</t>
+          <t>Wednesday 15 October 2025 11:00am</t>
         </is>
       </c>
       <c r="L189" s="1" t="n">
-        <v>45840.45833333334</v>
+        <v>45945.45833333334</v>
       </c>
       <c r="M189" t="inlineStr">
         <is>
-          <t>£35,000</t>
+          <t>£500,000</t>
         </is>
       </c>
       <c r="N189" s="1" t="n">
@@ -11360,12 +11422,12 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>Innovate UK innovation loans future economy: Round 21</t>
+          <t>Accelerated Knowledge Transfer 4 (AKT4) Addiction</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2188/overview/20c89a26-2479-4f80-b35a-b62ed3b9b3ce</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2178/overview/2699060f-dd6f-415b-ae47-bead15aa430e</t>
         </is>
       </c>
       <c r="D190" t="inlineStr">
@@ -11395,7 +11457,7 @@
       </c>
       <c r="M190" t="inlineStr">
         <is>
-          <t>£2.0 million</t>
+          <t>£35,000</t>
         </is>
       </c>
       <c r="N190" s="1" t="n">
@@ -11410,12 +11472,12 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>Farming Futures R&amp;D Fund: Precision Breeding Competition</t>
+          <t>Innovate UK innovation loans future economy: Round 21</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2168/overview/0fef9171-75b0-4f3e-acef-42920e7e5d5e</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2188/overview/20c89a26-2479-4f80-b35a-b62ed3b9b3ce</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
@@ -11437,15 +11499,15 @@
       <c r="J191" t="inlineStr"/>
       <c r="K191" t="inlineStr">
         <is>
-          <t>Wednesday 25 June 2025 11:00am</t>
+          <t>Wednesday 2 July 2025 11:00am</t>
         </is>
       </c>
       <c r="L191" s="1" t="n">
-        <v>45833.45833333334</v>
+        <v>45840.45833333334</v>
       </c>
       <c r="M191" t="inlineStr">
         <is>
-          <t>£2.5 million</t>
+          <t>£2.0 million</t>
         </is>
       </c>
       <c r="N191" s="1" t="n">
@@ -11460,12 +11522,12 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>Farming Futures R&amp;D Fund: low emissions farming</t>
+          <t>Farming Futures R&amp;D Fund: Precision Breeding Competition</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2169/overview/64b0d550-3f46-4ab4-a0cd-5fa7ac488cb6</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2168/overview/0fef9171-75b0-4f3e-acef-42920e7e5d5e</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
@@ -11510,12 +11572,12 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>Investor Partnerships: Clean Energy and Climate Technologies</t>
+          <t>Farming Futures R&amp;D Fund: low emissions farming</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2175/overview/7487b4f1-51e6-4f15-a4c8-f103559d14bb</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2169/overview/64b0d550-3f46-4ab4-a0cd-5fa7ac488cb6</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
@@ -11537,15 +11599,15 @@
       <c r="J193" t="inlineStr"/>
       <c r="K193" t="inlineStr">
         <is>
-          <t>Wednesday 2 July 2025 11:00am</t>
+          <t>Wednesday 25 June 2025 11:00am</t>
         </is>
       </c>
       <c r="L193" s="1" t="n">
-        <v>45840.45833333334</v>
+        <v>45833.45833333334</v>
       </c>
       <c r="M193" t="inlineStr">
         <is>
-          <t>£2.0 million</t>
+          <t>£2.5 million</t>
         </is>
       </c>
       <c r="N193" s="1" t="n">
@@ -11560,12 +11622,12 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>Full ADOPT Grant: Round 1</t>
+          <t>Investor Partnerships: Clean Energy and Climate Technologies</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2162/overview/c35de0a9-5072-4142-8a52-1cdce8ef3871</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2175/overview/7487b4f1-51e6-4f15-a4c8-f103559d14bb</t>
         </is>
       </c>
       <c r="D194" t="inlineStr">
@@ -11587,15 +11649,15 @@
       <c r="J194" t="inlineStr"/>
       <c r="K194" t="inlineStr">
         <is>
-          <t>Wednesday 25 June 2025 11:00am</t>
+          <t>Wednesday 2 July 2025 11:00am</t>
         </is>
       </c>
       <c r="L194" s="1" t="n">
-        <v>45833.45833333334</v>
+        <v>45840.45833333334</v>
       </c>
       <c r="M194" t="inlineStr">
         <is>
-          <t>£100,000</t>
+          <t>£2.0 million</t>
         </is>
       </c>
       <c r="N194" s="1" t="n">
@@ -11610,12 +11672,12 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>Horizon Europe Guarantee - EIT KICs 2023</t>
+          <t>Full ADOPT Grant: Round 1</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/1585/overview/32135a71-171a-46bf-ad56-e2e65a1a3574</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2162/overview/c35de0a9-5072-4142-8a52-1cdce8ef3871</t>
         </is>
       </c>
       <c r="D195" t="inlineStr">
@@ -11637,11 +11699,17 @@
       <c r="J195" t="inlineStr"/>
       <c r="K195" t="inlineStr">
         <is>
-          <t>Thursday 27 November 2025 4:00pm</t>
-        </is>
-      </c>
-      <c r="L195" t="inlineStr"/>
-      <c r="M195" t="inlineStr"/>
+          <t>Wednesday 25 June 2025 11:00am</t>
+        </is>
+      </c>
+      <c r="L195" s="1" t="n">
+        <v>45833.45833333334</v>
+      </c>
+      <c r="M195" t="inlineStr">
+        <is>
+          <t>£100,000</t>
+        </is>
+      </c>
       <c r="N195" s="1" t="n">
         <v>45819</v>
       </c>
@@ -11654,12 +11722,12 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>Horizon Europe Guarantee Extension</t>
+          <t>Horizon Europe Guarantee - EIT KICs 2023</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/1389/overview/b900fdc4-c48d-4d8a-8733-ce4ca210ae9a</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/1585/overview/32135a71-171a-46bf-ad56-e2e65a1a3574</t>
         </is>
       </c>
       <c r="D196" t="inlineStr">
@@ -11698,21 +11766,21 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>Knowledge Transfer Partnership (KTP): 2025 – 2026 Round 3</t>
+          <t>Horizon Europe Guarantee Extension</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2184/overview/c599b17c-e13a-4e13-995e-53cc4d4508a1</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/1389/overview/b900fdc4-c48d-4d8a-8733-ce4ca210ae9a</t>
         </is>
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>2025-06-16 22:04</t>
+          <t>2025-06-14 08:41</t>
         </is>
       </c>
       <c r="E197" s="1" t="n">
-        <v>45824.91944444444</v>
+        <v>45822.36180555556</v>
       </c>
       <c r="F197" t="b">
         <v>1</v>
@@ -11725,17 +11793,11 @@
       <c r="J197" t="inlineStr"/>
       <c r="K197" t="inlineStr">
         <is>
-          <t>Wednesday 17 September 2025 11:00am</t>
-        </is>
-      </c>
-      <c r="L197" s="1" t="n">
-        <v>45917.45833333334</v>
-      </c>
-      <c r="M197" t="inlineStr">
-        <is>
-          <t>£8,500</t>
-        </is>
-      </c>
+          <t>Thursday 27 November 2025 4:00pm</t>
+        </is>
+      </c>
+      <c r="L197" t="inlineStr"/>
+      <c r="M197" t="inlineStr"/>
       <c r="N197" s="1" t="n">
         <v>45819</v>
       </c>
@@ -11748,21 +11810,21 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>Agri-tech and food technology, Mid and North Wales - CRD</t>
+          <t>Knowledge Transfer Partnership (KTP): 2025 – 2026 Round 3</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2212/overview/4411087f-2a92-4aed-b735-d1a813376bec</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2184/overview/c599b17c-e13a-4e13-995e-53cc4d4508a1</t>
         </is>
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>2025-06-26 08:52</t>
+          <t>2025-06-16 22:04</t>
         </is>
       </c>
       <c r="E198" s="1" t="n">
-        <v>45834.36944444444</v>
+        <v>45824.91944444444</v>
       </c>
       <c r="F198" t="b">
         <v>1</v>
@@ -11775,19 +11837,19 @@
       <c r="J198" t="inlineStr"/>
       <c r="K198" t="inlineStr">
         <is>
-          <t>Wednesday 20 August 2025 11:00am</t>
+          <t>Wednesday 17 September 2025 11:00am</t>
         </is>
       </c>
       <c r="L198" s="1" t="n">
-        <v>45889.45833333334</v>
+        <v>45917.45833333334</v>
       </c>
       <c r="M198" t="inlineStr">
         <is>
-          <t>£500,000</t>
+          <t>£8,500</t>
         </is>
       </c>
       <c r="N198" s="1" t="n">
-        <v>45833</v>
+        <v>45819</v>
       </c>
     </row>
     <row r="199">
@@ -11798,12 +11860,12 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>Full ADOPT Grant Round 2</t>
+          <t>Agri-tech and food technology, Mid and North Wales - CRD</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2222/overview/c3d5b2f9-e4d4-4ddc-99a2-589904ac3d42</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2212/overview/4411087f-2a92-4aed-b735-d1a813376bec</t>
         </is>
       </c>
       <c r="D199" t="inlineStr">
@@ -11833,7 +11895,7 @@
       </c>
       <c r="M199" t="inlineStr">
         <is>
-          <t>£100,000</t>
+          <t>£500,000</t>
         </is>
       </c>
       <c r="N199" s="1" t="n">
@@ -11848,21 +11910,21 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>Innovate UK Innovation Loans Round 22</t>
+          <t>Full ADOPT Grant Round 2</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2236/overview/70cbae59-4e67-4626-8cb0-6bbbfc0cf6b7</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2222/overview/c3d5b2f9-e4d4-4ddc-99a2-589904ac3d42</t>
         </is>
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>2025-07-03 08:52</t>
+          <t>2025-06-26 08:52</t>
         </is>
       </c>
       <c r="E200" s="1" t="n">
-        <v>45841.36944444444</v>
+        <v>45834.36944444444</v>
       </c>
       <c r="F200" t="b">
         <v>1</v>
@@ -11875,19 +11937,19 @@
       <c r="J200" t="inlineStr"/>
       <c r="K200" t="inlineStr">
         <is>
-          <t>Wednesday 27 August 2025 11:00am</t>
+          <t>Wednesday 20 August 2025 11:00am</t>
         </is>
       </c>
       <c r="L200" s="1" t="n">
-        <v>45896.45833333334</v>
+        <v>45889.45833333334</v>
       </c>
       <c r="M200" t="inlineStr">
         <is>
-          <t>£5.0 million</t>
+          <t>£100,000</t>
         </is>
       </c>
       <c r="N200" s="1" t="n">
-        <v>45840</v>
+        <v>45833</v>
       </c>
     </row>
     <row r="201">
@@ -11898,21 +11960,21 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>Growth Catalyst Early Stage: New Innovators</t>
+          <t>Innovate UK Innovation Loans Round 22</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2220/overview/bcfd2780-f307-4434-be32-46889a239024</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2236/overview/70cbae59-4e67-4626-8cb0-6bbbfc0cf6b7</t>
         </is>
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>2025-07-07 08:54</t>
+          <t>2025-07-03 08:52</t>
         </is>
       </c>
       <c r="E201" s="1" t="n">
-        <v>45845.37083333333</v>
+        <v>45841.36944444444</v>
       </c>
       <c r="F201" t="b">
         <v>1</v>
@@ -11925,15 +11987,15 @@
       <c r="J201" t="inlineStr"/>
       <c r="K201" t="inlineStr">
         <is>
-          <t>Wednesday 6 August 2025 11:00am</t>
+          <t>Wednesday 27 August 2025 11:00am</t>
         </is>
       </c>
       <c r="L201" s="1" t="n">
-        <v>45875.45833333334</v>
+        <v>45896.45833333334</v>
       </c>
       <c r="M201" t="inlineStr">
         <is>
-          <t>£50,000</t>
+          <t>£5.0 million</t>
         </is>
       </c>
       <c r="N201" s="1" t="n">
@@ -11948,12 +12010,12 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>ATI Programme strategic batch: EoI – July 2025</t>
+          <t>Growth Catalyst Early Stage: New Innovators</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2228/overview/5ccf059d-ae66-4f72-a319-4b12cbd46d1c</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2220/overview/bcfd2780-f307-4434-be32-46889a239024</t>
         </is>
       </c>
       <c r="D202" t="inlineStr">
@@ -11975,13 +12037,17 @@
       <c r="J202" t="inlineStr"/>
       <c r="K202" t="inlineStr">
         <is>
-          <t>Wednesday 23 July 2025 11:00am</t>
+          <t>Wednesday 6 August 2025 11:00am</t>
         </is>
       </c>
       <c r="L202" s="1" t="n">
-        <v>45861.45833333334</v>
-      </c>
-      <c r="M202" t="inlineStr"/>
+        <v>45875.45833333334</v>
+      </c>
+      <c r="M202" t="inlineStr">
+        <is>
+          <t>£50,000</t>
+        </is>
+      </c>
       <c r="N202" s="1" t="n">
         <v>45840</v>
       </c>
@@ -11994,21 +12060,21 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>Contracts for Innovation: Resource Efficient Construction Impacts</t>
+          <t>ATI Programme strategic batch: EoI – July 2025</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2242/overview/51b1338a-0d60-43de-b062-fe7a48a7d42f</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2228/overview/5ccf059d-ae66-4f72-a319-4b12cbd46d1c</t>
         </is>
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>2025-07-09 08:54</t>
+          <t>2025-07-07 08:54</t>
         </is>
       </c>
       <c r="E203" s="1" t="n">
-        <v>45847.37083333333</v>
+        <v>45845.37083333333</v>
       </c>
       <c r="F203" t="b">
         <v>1</v>
@@ -12021,19 +12087,15 @@
       <c r="J203" t="inlineStr"/>
       <c r="K203" t="inlineStr">
         <is>
-          <t>Wednesday 27 August 2025 11:00am</t>
+          <t>Wednesday 23 July 2025 11:00am</t>
         </is>
       </c>
       <c r="L203" s="1" t="n">
-        <v>45896.45833333334</v>
-      </c>
-      <c r="M203" t="inlineStr">
-        <is>
-          <t>£300,000</t>
-        </is>
-      </c>
+        <v>45861.45833333334</v>
+      </c>
+      <c r="M203" t="inlineStr"/>
       <c r="N203" s="1" t="n">
-        <v>45847</v>
+        <v>45840</v>
       </c>
     </row>
     <row r="204">
@@ -12044,12 +12106,12 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>Contracts for Innovation: Resource Efficient Chemicals Impacts</t>
+          <t>Contracts for Innovation: Resource Efficient Construction Impacts</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2240/overview/10f28eca-01f0-4abf-8e0c-998151fe747b</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2242/overview/51b1338a-0d60-43de-b062-fe7a48a7d42f</t>
         </is>
       </c>
       <c r="D204" t="inlineStr">
@@ -12094,12 +12156,12 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>Contracts for Innovation: Resource Efficient Automotive Impacts</t>
+          <t>Contracts for Innovation: Resource Efficient Chemicals Impacts</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2241/overview/baec7aff-ca8b-456c-9e4d-d6eb9621a988</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2240/overview/10f28eca-01f0-4abf-8e0c-998151fe747b</t>
         </is>
       </c>
       <c r="D205" t="inlineStr">
@@ -12144,12 +12206,12 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>Future Flight: Regional Demonstrator 2</t>
+          <t>Contracts for Innovation: Resource Efficient Automotive Impacts</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2239/overview/7c5a9acd-4b31-414a-8e35-20dd1df3a2a1</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2241/overview/baec7aff-ca8b-456c-9e4d-d6eb9621a988</t>
         </is>
       </c>
       <c r="D206" t="inlineStr">
@@ -12171,15 +12233,15 @@
       <c r="J206" t="inlineStr"/>
       <c r="K206" t="inlineStr">
         <is>
-          <t>Thursday 17 July 2025 11:00am</t>
+          <t>Wednesday 27 August 2025 11:00am</t>
         </is>
       </c>
       <c r="L206" s="1" t="n">
-        <v>45855.45833333334</v>
+        <v>45896.45833333334</v>
       </c>
       <c r="M206" t="inlineStr">
         <is>
-          <t>£200,000</t>
+          <t>£300,000</t>
         </is>
       </c>
       <c r="N206" s="1" t="n">
@@ -12194,21 +12256,21 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>DRIVE35 Scale-up: Feasibility Studies</t>
+          <t>Future Flight: Regional Demonstrator 2</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2247/overview/53da287a-c141-48d2-a3eb-f854e14c6578</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2239/overview/7c5a9acd-4b31-414a-8e35-20dd1df3a2a1</t>
         </is>
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>2025-07-15 08:20</t>
+          <t>2025-07-09 08:54</t>
         </is>
       </c>
       <c r="E207" s="1" t="n">
-        <v>45853.34722222222</v>
+        <v>45847.37083333333</v>
       </c>
       <c r="F207" t="b">
         <v>1</v>
@@ -12221,15 +12283,15 @@
       <c r="J207" t="inlineStr"/>
       <c r="K207" t="inlineStr">
         <is>
-          <t>Wednesday 3 September 2025 11:00am</t>
+          <t>Thursday 17 July 2025 11:00am</t>
         </is>
       </c>
       <c r="L207" s="1" t="n">
-        <v>45903.45833333334</v>
+        <v>45855.45833333334</v>
       </c>
       <c r="M207" t="inlineStr">
         <is>
-          <t>£750,000</t>
+          <t>£200,000</t>
         </is>
       </c>
       <c r="N207" s="1" t="n">
@@ -12244,12 +12306,12 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>DRIVE35 Innovation Fund: Demonstrate</t>
+          <t>DRIVE35 Scale-up: Feasibility Studies</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2245/overview/777781a3-f181-42b3-a05e-86b96754f28d</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2247/overview/53da287a-c141-48d2-a3eb-f854e14c6578</t>
         </is>
       </c>
       <c r="D208" t="inlineStr">
@@ -12271,15 +12333,15 @@
       <c r="J208" t="inlineStr"/>
       <c r="K208" t="inlineStr">
         <is>
-          <t>Wednesday 1 October 2025 11:00am</t>
+          <t>Wednesday 3 September 2025 11:00am</t>
         </is>
       </c>
       <c r="L208" s="1" t="n">
-        <v>45931.45833333334</v>
+        <v>45903.45833333334</v>
       </c>
       <c r="M208" t="inlineStr">
         <is>
-          <t>£1.5 million</t>
+          <t>£750,000</t>
         </is>
       </c>
       <c r="N208" s="1" t="n">
@@ -12294,12 +12356,12 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>DRIVE35 Innovation Fund: Collaborate</t>
+          <t>DRIVE35 Innovation Fund: Demonstrate</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2244/overview/84f81488-4936-4551-a315-7ec40cf1065d</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2245/overview/777781a3-f181-42b3-a05e-86b96754f28d</t>
         </is>
       </c>
       <c r="D209" t="inlineStr">
@@ -12329,7 +12391,7 @@
       </c>
       <c r="M209" t="inlineStr">
         <is>
-          <t>£25.0 million</t>
+          <t>£1.5 million</t>
         </is>
       </c>
       <c r="N209" s="1" t="n">
@@ -12344,21 +12406,21 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>ADOPT Facilitator Support Grant: Round 3</t>
+          <t>DRIVE35 Innovation Fund: Collaborate</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2251/overview/f40e861a-c7f6-4597-ac5d-2e8d1b4f59f8</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2244/overview/84f81488-4936-4551-a315-7ec40cf1065d</t>
         </is>
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>2025-07-25 08:20</t>
+          <t>2025-07-15 08:20</t>
         </is>
       </c>
       <c r="E210" s="1" t="n">
-        <v>45863.34722222222</v>
+        <v>45853.34722222222</v>
       </c>
       <c r="F210" t="b">
         <v>1</v>
@@ -12371,19 +12433,19 @@
       <c r="J210" t="inlineStr"/>
       <c r="K210" t="inlineStr">
         <is>
-          <t>Wednesday 3 September 2025 11:00am</t>
+          <t>Wednesday 1 October 2025 11:00am</t>
         </is>
       </c>
       <c r="L210" s="1" t="n">
-        <v>45903.45833333334</v>
+        <v>45931.45833333334</v>
       </c>
       <c r="M210" t="inlineStr">
         <is>
-          <t>£2,500</t>
+          <t>£25.0 million</t>
         </is>
       </c>
       <c r="N210" s="1" t="n">
-        <v>45861</v>
+        <v>45847</v>
       </c>
     </row>
     <row r="211">
@@ -12394,21 +12456,21 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>Sovereign AI - Proof of concept</t>
+          <t>ADOPT Facilitator Support Grant: Round 3</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2259/overview/9061ddb2-fa12-45c9-8691-d36649c96e9c</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2251/overview/f40e861a-c7f6-4597-ac5d-2e8d1b4f59f8</t>
         </is>
       </c>
       <c r="D211" t="inlineStr">
         <is>
-          <t>2025-08-07 08:21</t>
+          <t>2025-07-25 08:20</t>
         </is>
       </c>
       <c r="E211" s="1" t="n">
-        <v>45876.34791666667</v>
+        <v>45863.34722222222</v>
       </c>
       <c r="F211" t="b">
         <v>1</v>
@@ -12421,19 +12483,19 @@
       <c r="J211" t="inlineStr"/>
       <c r="K211" t="inlineStr">
         <is>
-          <t>Wednesday 10 September 2025 11:00am</t>
+          <t>Wednesday 3 September 2025 11:00am</t>
         </is>
       </c>
       <c r="L211" s="1" t="n">
-        <v>45910.45833333334</v>
+        <v>45903.45833333334</v>
       </c>
       <c r="M211" t="inlineStr">
         <is>
-          <t>£120,000</t>
+          <t>£2,500</t>
         </is>
       </c>
       <c r="N211" s="1" t="n">
-        <v>45875</v>
+        <v>45861</v>
       </c>
     </row>
     <row r="212">
@@ -12444,21 +12506,21 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>Obesity Pathway Innovation Programme (OPIP): Strand 3</t>
+          <t>Sovereign AI - Proof of concept</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2186/overview/e51c18bc-21b3-450d-bdbc-2f43dad3b268</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2259/overview/9061ddb2-fa12-45c9-8691-d36649c96e9c</t>
         </is>
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t>2025-08-14 08:20</t>
+          <t>2025-08-07 08:21</t>
         </is>
       </c>
       <c r="E212" s="1" t="n">
-        <v>45883.34722222222</v>
+        <v>45876.34791666667</v>
       </c>
       <c r="F212" t="b">
         <v>1</v>
@@ -12471,19 +12533,19 @@
       <c r="J212" t="inlineStr"/>
       <c r="K212" t="inlineStr">
         <is>
-          <t>Wednesday 19 November 2025 11:00am</t>
+          <t>Wednesday 10 September 2025 11:00am</t>
         </is>
       </c>
       <c r="L212" s="1" t="n">
-        <v>45980.45833333334</v>
+        <v>45910.45833333334</v>
       </c>
       <c r="M212" t="inlineStr">
         <is>
-          <t>£8.0 million</t>
+          <t>£120,000</t>
         </is>
       </c>
       <c r="N212" s="1" t="n">
-        <v>45882</v>
+        <v>45875</v>
       </c>
     </row>
     <row r="213">
@@ -12494,12 +12556,12 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>Obesity Pathway Innovation Programme (OPIP): Strand 2</t>
+          <t>Obesity Pathway Innovation Programme (OPIP): Strand 3</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2185/overview/d5b2aeb3-c2e4-4d78-9be3-f1d9919b0956</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2186/overview/e51c18bc-21b3-450d-bdbc-2f43dad3b268</t>
         </is>
       </c>
       <c r="D213" t="inlineStr">
@@ -12529,7 +12591,7 @@
       </c>
       <c r="M213" t="inlineStr">
         <is>
-          <t>£4.5 million</t>
+          <t>£8.0 million</t>
         </is>
       </c>
       <c r="N213" s="1" t="n">
@@ -12544,12 +12606,12 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>Obesity Pathway Innovation Programme (OPIP): Strand 1</t>
+          <t>Obesity Pathway Innovation Programme (OPIP): Strand 2</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2177/overview/696c1e3c-589d-4c37-8958-6255d1dc125a</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2185/overview/d5b2aeb3-c2e4-4d78-9be3-f1d9919b0956</t>
         </is>
       </c>
       <c r="D214" t="inlineStr">
@@ -12579,7 +12641,7 @@
       </c>
       <c r="M214" t="inlineStr">
         <is>
-          <t>£3.5 million</t>
+          <t>£4.5 million</t>
         </is>
       </c>
       <c r="N214" s="1" t="n">
@@ -12594,21 +12656,21 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>Analysis for Innovators: National Physical Laboratory Stage 1</t>
+          <t>Obesity Pathway Innovation Programme (OPIP): Strand 1</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2266/overview/2fcad3ee-b5d6-4f01-8b1a-0e1af3c93023</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2177/overview/696c1e3c-589d-4c37-8958-6255d1dc125a</t>
         </is>
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>2025-08-26 08:20</t>
+          <t>2025-08-14 08:20</t>
         </is>
       </c>
       <c r="E215" s="1" t="n">
-        <v>45895.34722222222</v>
+        <v>45883.34722222222</v>
       </c>
       <c r="F215" t="b">
         <v>1</v>
@@ -12621,19 +12683,19 @@
       <c r="J215" t="inlineStr"/>
       <c r="K215" t="inlineStr">
         <is>
-          <t>Wednesday 10 September 2025 11:00am</t>
+          <t>Wednesday 19 November 2025 11:00am</t>
         </is>
       </c>
       <c r="L215" s="1" t="n">
-        <v>45910.45833333334</v>
+        <v>45980.45833333334</v>
       </c>
       <c r="M215" t="inlineStr">
         <is>
-          <t>£100,000</t>
+          <t>£3.5 million</t>
         </is>
       </c>
       <c r="N215" s="1" t="n">
-        <v>45889</v>
+        <v>45882</v>
       </c>
     </row>
     <row r="216">
@@ -12644,21 +12706,21 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>Full ADOPT Grant Round 3</t>
+          <t>Analysis for Innovators: National Physical Laboratory Stage 1</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2265/overview/fae182db-d9e5-4173-bb59-8fde361ccad4</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2266/overview/2fcad3ee-b5d6-4f01-8b1a-0e1af3c93023</t>
         </is>
       </c>
       <c r="D216" t="inlineStr">
         <is>
-          <t>2025-08-27 08:18</t>
+          <t>2025-08-26 08:20</t>
         </is>
       </c>
       <c r="E216" s="1" t="n">
-        <v>45896.34583333333</v>
+        <v>45895.34722222222</v>
       </c>
       <c r="F216" t="b">
         <v>1</v>
@@ -12671,11 +12733,11 @@
       <c r="J216" t="inlineStr"/>
       <c r="K216" t="inlineStr">
         <is>
-          <t>Wednesday 15 October 2025 11:00am</t>
+          <t>Wednesday 10 September 2025 11:00am</t>
         </is>
       </c>
       <c r="L216" s="1" t="n">
-        <v>45945.45833333334</v>
+        <v>45910.45833333334</v>
       </c>
       <c r="M216" t="inlineStr">
         <is>
@@ -12683,7 +12745,7 @@
         </is>
       </c>
       <c r="N216" s="1" t="n">
-        <v>45896</v>
+        <v>45889</v>
       </c>
     </row>
     <row r="217">
@@ -12694,21 +12756,21 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>ATI Programme strategic batch: EoI – September 2025</t>
+          <t>Full ADOPT Grant Round 3</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2273/overview/b30df196-a9a2-4e53-85e1-e3e6aaa5c5b7</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2265/overview/fae182db-d9e5-4173-bb59-8fde361ccad4</t>
         </is>
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>2025-09-01 08:20</t>
+          <t>2025-08-27 08:18</t>
         </is>
       </c>
       <c r="E217" s="1" t="n">
-        <v>45901.34722222222</v>
+        <v>45896.34583333333</v>
       </c>
       <c r="F217" t="b">
         <v>1</v>
@@ -12721,13 +12783,17 @@
       <c r="J217" t="inlineStr"/>
       <c r="K217" t="inlineStr">
         <is>
-          <t>Wednesday 17 September 2025 11:00am</t>
+          <t>Wednesday 15 October 2025 11:00am</t>
         </is>
       </c>
       <c r="L217" s="1" t="n">
-        <v>45917.45833333334</v>
-      </c>
-      <c r="M217" t="inlineStr"/>
+        <v>45945.45833333334</v>
+      </c>
+      <c r="M217" t="inlineStr">
+        <is>
+          <t>£100,000</t>
+        </is>
+      </c>
       <c r="N217" s="1" t="n">
         <v>45896</v>
       </c>
@@ -12740,21 +12806,21 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>Farming Innovation Programme: Small R&amp;D Partnership Projects Rd 4</t>
+          <t>ATI Programme strategic batch: EoI – September 2025</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2010/overview/bcd5cf06-313c-4197-ae47-0035f674717f</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2273/overview/b30df196-a9a2-4e53-85e1-e3e6aaa5c5b7</t>
         </is>
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>2025-09-02 08:19</t>
+          <t>2025-09-01 08:20</t>
         </is>
       </c>
       <c r="E218" s="1" t="n">
-        <v>45902.34652777778</v>
+        <v>45901.34722222222</v>
       </c>
       <c r="F218" t="b">
         <v>1</v>
@@ -12767,17 +12833,13 @@
       <c r="J218" t="inlineStr"/>
       <c r="K218" t="inlineStr">
         <is>
-          <t>Wednesday 5 November 2025 11:00am</t>
+          <t>Wednesday 17 September 2025 11:00am</t>
         </is>
       </c>
       <c r="L218" s="1" t="n">
-        <v>45966.45833333334</v>
-      </c>
-      <c r="M218" t="inlineStr">
-        <is>
-          <t>£3.0 million</t>
-        </is>
-      </c>
+        <v>45917.45833333334</v>
+      </c>
+      <c r="M218" t="inlineStr"/>
       <c r="N218" s="1" t="n">
         <v>45896</v>
       </c>
@@ -12790,21 +12852,21 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>ADOPT Facilitator Support Grant: Round 4</t>
+          <t>Farming Innovation Programme: Small R&amp;D Partnership Projects Rd 4</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2277/overview/7386173a-c074-4617-b7d0-f54f3a458247</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2010/overview/bcd5cf06-313c-4197-ae47-0035f674717f</t>
         </is>
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>2025-09-04 08:18</t>
+          <t>2025-09-02 08:19</t>
         </is>
       </c>
       <c r="E219" s="1" t="n">
-        <v>45904.34583333333</v>
+        <v>45902.34652777778</v>
       </c>
       <c r="F219" t="b">
         <v>1</v>
@@ -12817,19 +12879,19 @@
       <c r="J219" t="inlineStr"/>
       <c r="K219" t="inlineStr">
         <is>
-          <t>Wednesday 15 October 2025 11:00am</t>
+          <t>Wednesday 5 November 2025 11:00am</t>
         </is>
       </c>
       <c r="L219" s="1" t="n">
-        <v>45945.45833333334</v>
+        <v>45966.45833333334</v>
       </c>
       <c r="M219" t="inlineStr">
         <is>
-          <t>£2,500</t>
+          <t>£3.0 million</t>
         </is>
       </c>
       <c r="N219" s="1" t="n">
-        <v>45903</v>
+        <v>45896</v>
       </c>
     </row>
     <row r="220">
@@ -12840,21 +12902,21 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>Innovate UK Innovation Loans Round 23</t>
+          <t>ADOPT Facilitator Support Grant: Round 4</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2275/overview/dec9b656-5f30-414e-a169-e11e17d04896</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2277/overview/7386173a-c074-4617-b7d0-f54f3a458247</t>
         </is>
       </c>
       <c r="D220" t="inlineStr">
         <is>
-          <t>2025-09-05 08:18</t>
+          <t>2025-09-04 08:18</t>
         </is>
       </c>
       <c r="E220" s="1" t="n">
-        <v>45905.34583333333</v>
+        <v>45904.34583333333</v>
       </c>
       <c r="F220" t="b">
         <v>1</v>
@@ -12867,15 +12929,15 @@
       <c r="J220" t="inlineStr"/>
       <c r="K220" t="inlineStr">
         <is>
-          <t>Wednesday 22 October 2025 11:00am</t>
+          <t>Wednesday 15 October 2025 11:00am</t>
         </is>
       </c>
       <c r="L220" s="1" t="n">
-        <v>45952.45833333334</v>
+        <v>45945.45833333334</v>
       </c>
       <c r="M220" t="inlineStr">
         <is>
-          <t>£5.0 million</t>
+          <t>£2,500</t>
         </is>
       </c>
       <c r="N220" s="1" t="n">
@@ -12890,21 +12952,21 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>UK-Netherlands Co-Innovation and Testbeds Pilot for Quantum Tech</t>
+          <t>Innovate UK Innovation Loans Round 23</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2288/overview/d547d84e-d652-4ed6-9c85-b12ab8d785d2</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2275/overview/dec9b656-5f30-414e-a169-e11e17d04896</t>
         </is>
       </c>
       <c r="D221" t="inlineStr">
         <is>
-          <t>2025-09-12 08:17</t>
+          <t>2025-09-05 08:18</t>
         </is>
       </c>
       <c r="E221" s="1" t="n">
-        <v>45912.34513888889</v>
+        <v>45905.34583333333</v>
       </c>
       <c r="F221" t="b">
         <v>1</v>
@@ -12917,19 +12979,19 @@
       <c r="J221" t="inlineStr"/>
       <c r="K221" t="inlineStr">
         <is>
-          <t>Tuesday 28 October 2025 11:00am</t>
+          <t>Wednesday 22 October 2025 11:00am</t>
         </is>
       </c>
       <c r="L221" s="1" t="n">
-        <v>45958.45833333334</v>
+        <v>45952.45833333334</v>
       </c>
       <c r="M221" t="inlineStr">
         <is>
-          <t>£300,000</t>
+          <t>£5.0 million</t>
         </is>
       </c>
       <c r="N221" s="1" t="n">
-        <v>45910</v>
+        <v>45903</v>
       </c>
     </row>
     <row r="222">
@@ -12940,21 +13002,21 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>Contracts for Innovation: Quantum Technologies for Transport - Phase 1</t>
+          <t>UK-Netherlands Co-Innovation and Testbeds Pilot for Quantum Tech</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2292/overview/cdea3182-7495-4cad-8435-f49882f08ec7</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2288/overview/d547d84e-d652-4ed6-9c85-b12ab8d785d2</t>
         </is>
       </c>
       <c r="D222" t="inlineStr">
         <is>
-          <t>2025-09-16 08:19</t>
+          <t>2025-09-12 08:17</t>
         </is>
       </c>
       <c r="E222" s="1" t="n">
-        <v>45916.34652777778</v>
+        <v>45912.34513888889</v>
       </c>
       <c r="F222" t="b">
         <v>1</v>
@@ -12967,15 +13029,15 @@
       <c r="J222" t="inlineStr"/>
       <c r="K222" t="inlineStr">
         <is>
-          <t>Wednesday 15 October 2025 11:00am</t>
+          <t>Tuesday 28 October 2025 11:00am</t>
         </is>
       </c>
       <c r="L222" s="1" t="n">
-        <v>45945.45833333334</v>
+        <v>45958.45833333334</v>
       </c>
       <c r="M222" t="inlineStr">
         <is>
-          <t>£40,000</t>
+          <t>£300,000</t>
         </is>
       </c>
       <c r="N222" s="1" t="n">
@@ -12990,21 +13052,21 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>DRIVE35 Scale-up Fund</t>
+          <t>Contracts for Innovation: Quantum Technologies for Transport - Phase 1</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2279/overview/029bd996-9abd-42d9-8134-e2d34e3cfff5</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2292/overview/cdea3182-7495-4cad-8435-f49882f08ec7</t>
         </is>
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>2025-09-17 08:18</t>
+          <t>2025-09-16 08:19</t>
         </is>
       </c>
       <c r="E223" s="1" t="n">
-        <v>45917.34583333333</v>
+        <v>45916.34652777778</v>
       </c>
       <c r="F223" t="b">
         <v>1</v>
@@ -13017,17 +13079,19 @@
       <c r="J223" t="inlineStr"/>
       <c r="K223" t="inlineStr">
         <is>
-          <t>There is no submission deadline</t>
-        </is>
-      </c>
-      <c r="L223" t="inlineStr"/>
+          <t>Wednesday 15 October 2025 11:00am</t>
+        </is>
+      </c>
+      <c r="L223" s="1" t="n">
+        <v>45945.45833333334</v>
+      </c>
       <c r="M223" t="inlineStr">
         <is>
-          <t>£20.0 million</t>
+          <t>£40,000</t>
         </is>
       </c>
       <c r="N223" s="1" t="n">
-        <v>45917</v>
+        <v>45910</v>
       </c>
     </row>
     <row r="224">
@@ -13038,21 +13102,21 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>Commercialising Knowledge Assets Fund (CKAF) Winter</t>
+          <t>DRIVE35 Scale-up Fund</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2295/overview/cdce9dab-263c-444b-9e91-61f13046bd62</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2279/overview/029bd996-9abd-42d9-8134-e2d34e3cfff5</t>
         </is>
       </c>
       <c r="D224" t="inlineStr">
         <is>
-          <t>2025-09-18 08:17</t>
+          <t>2025-09-17 08:18</t>
         </is>
       </c>
       <c r="E224" s="1" t="n">
-        <v>45918.34513888889</v>
+        <v>45917.34583333333</v>
       </c>
       <c r="F224" t="b">
         <v>1</v>
@@ -13065,15 +13129,13 @@
       <c r="J224" t="inlineStr"/>
       <c r="K224" t="inlineStr">
         <is>
-          <t>Thursday 4 December 2025 11:00am</t>
-        </is>
-      </c>
-      <c r="L224" s="1" t="n">
-        <v>45995.45833333334</v>
-      </c>
+          <t>There is no submission deadline</t>
+        </is>
+      </c>
+      <c r="L224" t="inlineStr"/>
       <c r="M224" t="inlineStr">
         <is>
-          <t>£250,000</t>
+          <t>£20.0 million</t>
         </is>
       </c>
       <c r="N224" s="1" t="n">
@@ -13088,21 +13150,21 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>Resource efficiency for resilience and sustainability FS</t>
+          <t>Commercialising Knowledge Assets Fund (CKAF) Winter</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2293/overview/2efee934-8622-4686-bc02-a6ac7fc9e5a6</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2295/overview/cdce9dab-263c-444b-9e91-61f13046bd62</t>
         </is>
       </c>
       <c r="D225" t="inlineStr">
         <is>
-          <t>2025-09-20 08:16</t>
+          <t>2025-09-18 08:17</t>
         </is>
       </c>
       <c r="E225" s="1" t="n">
-        <v>45920.34444444445</v>
+        <v>45918.34513888889</v>
       </c>
       <c r="F225" t="b">
         <v>1</v>
@@ -13115,15 +13177,15 @@
       <c r="J225" t="inlineStr"/>
       <c r="K225" t="inlineStr">
         <is>
-          <t>Monday 3 November 2025 11:00am</t>
+          <t>Thursday 4 December 2025 11:00am</t>
         </is>
       </c>
       <c r="L225" s="1" t="n">
-        <v>45964.45833333334</v>
+        <v>45995.45833333334</v>
       </c>
       <c r="M225" t="inlineStr">
         <is>
-          <t>£25,000</t>
+          <t>£250,000</t>
         </is>
       </c>
       <c r="N225" s="1" t="n">
@@ -13138,21 +13200,21 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>Ofgem Strategic Innovation Fund Round 5 Discovery C4</t>
+          <t>Resource efficiency for resilience and sustainability FS</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2284/overview/aa6bd2b1-f6e1-4e96-bd4c-0557c10779c8</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2293/overview/2efee934-8622-4686-bc02-a6ac7fc9e5a6</t>
         </is>
       </c>
       <c r="D226" t="inlineStr">
         <is>
-          <t>2025-09-23 08:18</t>
+          <t>2025-09-20 08:16</t>
         </is>
       </c>
       <c r="E226" s="1" t="n">
-        <v>45923.34583333333</v>
+        <v>45920.34444444445</v>
       </c>
       <c r="F226" t="b">
         <v>1</v>
@@ -13165,15 +13227,15 @@
       <c r="J226" t="inlineStr"/>
       <c r="K226" t="inlineStr">
         <is>
-          <t>Wednesday 22 October 2025 11:00am</t>
+          <t>Monday 3 November 2025 11:00am</t>
         </is>
       </c>
       <c r="L226" s="1" t="n">
-        <v>45952.45833333334</v>
+        <v>45964.45833333334</v>
       </c>
       <c r="M226" t="inlineStr">
         <is>
-          <t>£150,000</t>
+          <t>£25,000</t>
         </is>
       </c>
       <c r="N226" s="1" t="n">
@@ -13188,21 +13250,21 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>Farming Innovation Programme: Feasibility Round 4</t>
+          <t>Ofgem Strategic Innovation Fund Round 5 Discovery C4</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2006/overview/b67973b5-6d46-4a34-a864-bec1212e3fe0</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2284/overview/aa6bd2b1-f6e1-4e96-bd4c-0557c10779c8</t>
         </is>
       </c>
       <c r="D227" t="inlineStr">
         <is>
-          <t>2025-09-29 08:20</t>
+          <t>2025-09-23 08:18</t>
         </is>
       </c>
       <c r="E227" s="1" t="n">
-        <v>45929.34722222222</v>
+        <v>45923.34583333333</v>
       </c>
       <c r="F227" t="b">
         <v>1</v>
@@ -13215,19 +13277,19 @@
       <c r="J227" t="inlineStr"/>
       <c r="K227" t="inlineStr">
         <is>
-          <t>Wednesday 3 December 2025 11:00am</t>
+          <t>Wednesday 22 October 2025 11:00am</t>
         </is>
       </c>
       <c r="L227" s="1" t="n">
-        <v>45994.45833333334</v>
+        <v>45952.45833333334</v>
       </c>
       <c r="M227" t="inlineStr">
         <is>
-          <t>£500,000</t>
+          <t>£150,000</t>
         </is>
       </c>
       <c r="N227" s="1" t="n">
-        <v>45924</v>
+        <v>45917</v>
       </c>
     </row>
     <row r="228">
@@ -13238,21 +13300,21 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>Eureka GlobalStars Japan 2026</t>
+          <t>Farming Innovation Programme: Feasibility Round 4</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2276/overview/19635c62-dd91-41d8-a90e-547cdb5acbfa</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2006/overview/b67973b5-6d46-4a34-a864-bec1212e3fe0</t>
         </is>
       </c>
       <c r="D228" t="inlineStr">
         <is>
-          <t>2025-10-03 08:17</t>
+          <t>2025-09-29 08:20</t>
         </is>
       </c>
       <c r="E228" s="1" t="n">
-        <v>45933.34513888889</v>
+        <v>45929.34722222222</v>
       </c>
       <c r="F228" t="b">
         <v>1</v>
@@ -13265,19 +13327,19 @@
       <c r="J228" t="inlineStr"/>
       <c r="K228" t="inlineStr">
         <is>
-          <t>Wednesday 21 January 2026 11:00am</t>
+          <t>Wednesday 3 December 2025 11:00am</t>
         </is>
       </c>
       <c r="L228" s="1" t="n">
-        <v>46043.45833333334</v>
+        <v>45994.45833333334</v>
       </c>
       <c r="M228" t="inlineStr">
         <is>
-          <t>£600,000</t>
+          <t>£500,000</t>
         </is>
       </c>
       <c r="N228" s="1" t="n">
-        <v>45931</v>
+        <v>45924</v>
       </c>
     </row>
     <row r="229">
@@ -13288,21 +13350,21 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>CAM Pathfinder: Feasibility studies 2</t>
+          <t>Eureka GlobalStars Japan 2026</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2307/overview/8eec43e7-96a5-49d1-97e1-3400321160f9</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2276/overview/19635c62-dd91-41d8-a90e-547cdb5acbfa</t>
         </is>
       </c>
       <c r="D229" t="inlineStr">
         <is>
-          <t>2025-10-10 08:18</t>
+          <t>2025-10-03 08:17</t>
         </is>
       </c>
       <c r="E229" s="1" t="n">
-        <v>45940.34583333333</v>
+        <v>45933.34513888889</v>
       </c>
       <c r="F229" t="b">
         <v>1</v>
@@ -13315,19 +13377,19 @@
       <c r="J229" t="inlineStr"/>
       <c r="K229" t="inlineStr">
         <is>
-          <t>Wednesday 26 November 2025 11:00am</t>
+          <t>Wednesday 21 January 2026 11:00am</t>
         </is>
       </c>
       <c r="L229" s="1" t="n">
-        <v>45987.45833333334</v>
+        <v>46043.45833333334</v>
       </c>
       <c r="M229" t="inlineStr">
         <is>
-          <t>£250,000</t>
+          <t>£600,000</t>
         </is>
       </c>
       <c r="N229" s="1" t="n">
-        <v>45938</v>
+        <v>45931</v>
       </c>
     </row>
     <row r="230">
@@ -13338,21 +13400,21 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>ATI Programme strategic batch EoI – October 2025</t>
+          <t>CAM Pathfinder: Feasibility studies 2</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2317/overview/c946fbde-725e-4f85-bb3f-3219576c4a01</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2307/overview/8eec43e7-96a5-49d1-97e1-3400321160f9</t>
         </is>
       </c>
       <c r="D230" t="inlineStr">
         <is>
-          <t>2025-10-14 08:17</t>
+          <t>2025-10-10 08:18</t>
         </is>
       </c>
       <c r="E230" s="1" t="n">
-        <v>45944.34513888889</v>
+        <v>45940.34583333333</v>
       </c>
       <c r="F230" t="b">
         <v>1</v>
@@ -13365,13 +13427,17 @@
       <c r="J230" t="inlineStr"/>
       <c r="K230" t="inlineStr">
         <is>
-          <t>Wednesday 22 October 2025 11:00am</t>
+          <t>Wednesday 26 November 2025 11:00am</t>
         </is>
       </c>
       <c r="L230" s="1" t="n">
-        <v>45952.45833333334</v>
-      </c>
-      <c r="M230" t="inlineStr"/>
+        <v>45987.45833333334</v>
+      </c>
+      <c r="M230" t="inlineStr">
+        <is>
+          <t>£250,000</t>
+        </is>
+      </c>
       <c r="N230" s="1" t="n">
         <v>45938</v>
       </c>
@@ -13384,21 +13450,21 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>CAM Pathfinder: Enable</t>
+          <t>ATI Programme strategic batch EoI – October 2025</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2318/overview/39cd0e04-6f9c-40da-b0be-8eaae7f1603d</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2317/overview/c946fbde-725e-4f85-bb3f-3219576c4a01</t>
         </is>
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>2025-10-15 08:19</t>
+          <t>2025-10-14 08:17</t>
         </is>
       </c>
       <c r="E231" s="1" t="n">
-        <v>45945.34652777778</v>
+        <v>45944.34513888889</v>
       </c>
       <c r="F231" t="b">
         <v>1</v>
@@ -13411,19 +13477,15 @@
       <c r="J231" t="inlineStr"/>
       <c r="K231" t="inlineStr">
         <is>
-          <t>Wednesday 17 December 2025 11:00am</t>
+          <t>Wednesday 22 October 2025 11:00am</t>
         </is>
       </c>
       <c r="L231" s="1" t="n">
-        <v>46008.45833333334</v>
-      </c>
-      <c r="M231" t="inlineStr">
-        <is>
-          <t>£4.0 million</t>
-        </is>
-      </c>
+        <v>45952.45833333334</v>
+      </c>
+      <c r="M231" t="inlineStr"/>
       <c r="N231" s="1" t="n">
-        <v>45945</v>
+        <v>45938</v>
       </c>
     </row>
     <row r="232">
@@ -13434,12 +13496,12 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>CAM Pathfinder: Demonstrate</t>
+          <t>CAM Pathfinder: Enable</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2315/overview/f02885bb-e043-4a60-8d0c-22242bd77fa9</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2318/overview/39cd0e04-6f9c-40da-b0be-8eaae7f1603d</t>
         </is>
       </c>
       <c r="D232" t="inlineStr">
@@ -13469,7 +13531,7 @@
       </c>
       <c r="M232" t="inlineStr">
         <is>
-          <t>£2.0 million</t>
+          <t>£4.0 million</t>
         </is>
       </c>
       <c r="N232" s="1" t="n">
@@ -13484,21 +13546,21 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>Launchpad: life and health sciences, Northern Ireland – Rd3 MFA</t>
+          <t>CAM Pathfinder: Demonstrate</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2305/overview/fe565f48-36a8-4d8b-8515-e89d750f259c</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2315/overview/f02885bb-e043-4a60-8d0c-22242bd77fa9</t>
         </is>
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>2025-10-16 08:19</t>
+          <t>2025-10-15 08:19</t>
         </is>
       </c>
       <c r="E233" s="1" t="n">
-        <v>45946.34652777778</v>
+        <v>45945.34652777778</v>
       </c>
       <c r="F233" t="b">
         <v>1</v>
@@ -13511,15 +13573,15 @@
       <c r="J233" t="inlineStr"/>
       <c r="K233" t="inlineStr">
         <is>
-          <t>Wednesday 26 November 2025 11:00am</t>
+          <t>Wednesday 17 December 2025 11:00am</t>
         </is>
       </c>
       <c r="L233" s="1" t="n">
-        <v>45987.45833333334</v>
+        <v>46008.45833333334</v>
       </c>
       <c r="M233" t="inlineStr">
         <is>
-          <t>£100,000</t>
+          <t>£2.0 million</t>
         </is>
       </c>
       <c r="N233" s="1" t="n">
@@ -13534,21 +13596,21 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>ADOPT Facilitator Support Grant: Round 5</t>
+          <t>Launchpad: life and health sciences, Northern Ireland – Rd3 MFA</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2299/overview/0a26e49f-fa03-4096-aa8b-3eb39b68f20d</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2305/overview/fe565f48-36a8-4d8b-8515-e89d750f259c</t>
         </is>
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t>2025-10-17 08:19</t>
+          <t>2025-10-16 08:19</t>
         </is>
       </c>
       <c r="E234" s="1" t="n">
-        <v>45947.34652777778</v>
+        <v>45946.34652777778</v>
       </c>
       <c r="F234" t="b">
         <v>1</v>
@@ -13569,7 +13631,7 @@
       </c>
       <c r="M234" t="inlineStr">
         <is>
-          <t>£2,500</t>
+          <t>£100,000</t>
         </is>
       </c>
       <c r="N234" s="1" t="n">
@@ -13584,21 +13646,21 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>Battery Innovation Feasibility Studies Round 1</t>
+          <t>ADOPT Facilitator Support Grant: Round 5</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2313/overview/508ab35f-0e07-4e84-8e31-bbbcb619bc9e</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2299/overview/0a26e49f-fa03-4096-aa8b-3eb39b68f20d</t>
         </is>
       </c>
       <c r="D235" t="inlineStr">
         <is>
-          <t>2025-10-18 08:16</t>
+          <t>2025-10-17 08:19</t>
         </is>
       </c>
       <c r="E235" s="1" t="n">
-        <v>45948.34444444445</v>
+        <v>45947.34652777778</v>
       </c>
       <c r="F235" t="b">
         <v>1</v>
@@ -13611,15 +13673,15 @@
       <c r="J235" t="inlineStr"/>
       <c r="K235" t="inlineStr">
         <is>
-          <t>Wednesday 17 December 2025 11:00am</t>
+          <t>Wednesday 26 November 2025 11:00am</t>
         </is>
       </c>
       <c r="L235" s="1" t="n">
-        <v>46008.45833333334</v>
+        <v>45987.45833333334</v>
       </c>
       <c r="M235" t="inlineStr">
         <is>
-          <t>£500,000</t>
+          <t>£2,500</t>
         </is>
       </c>
       <c r="N235" s="1" t="n">
@@ -13634,12 +13696,12 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>Battery Innovation Concept Development Round 1</t>
+          <t>Battery Innovation Feasibility Studies Round 1</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2314/overview/4d1e65d7-b380-41b7-8dcf-b25cd26b9ab5</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2313/overview/508ab35f-0e07-4e84-8e31-bbbcb619bc9e</t>
         </is>
       </c>
       <c r="D236" t="inlineStr">
@@ -13669,7 +13731,7 @@
       </c>
       <c r="M236" t="inlineStr">
         <is>
-          <t>£4.0 million</t>
+          <t>£500,000</t>
         </is>
       </c>
       <c r="N236" s="1" t="n">
@@ -13684,21 +13746,21 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>The Agentic AI Pioneers Prize</t>
+          <t>Battery Innovation Concept Development Round 1</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2316/overview/fa0eeab0-3021-4cbc-8975-5bd45a7d642a</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2314/overview/4d1e65d7-b380-41b7-8dcf-b25cd26b9ab5</t>
         </is>
       </c>
       <c r="D237" t="inlineStr">
         <is>
-          <t>2025-10-21 08:20</t>
+          <t>2025-10-18 08:16</t>
         </is>
       </c>
       <c r="E237" s="1" t="n">
-        <v>45951.34722222222</v>
+        <v>45948.34444444445</v>
       </c>
       <c r="F237" t="b">
         <v>1</v>
@@ -13711,13 +13773,17 @@
       <c r="J237" t="inlineStr"/>
       <c r="K237" t="inlineStr">
         <is>
-          <t>Wednesday 19 November 2025 11:00am</t>
+          <t>Wednesday 17 December 2025 11:00am</t>
         </is>
       </c>
       <c r="L237" s="1" t="n">
-        <v>45980.45833333334</v>
-      </c>
-      <c r="M237" t="inlineStr"/>
+        <v>46008.45833333334</v>
+      </c>
+      <c r="M237" t="inlineStr">
+        <is>
+          <t>£4.0 million</t>
+        </is>
+      </c>
       <c r="N237" s="1" t="n">
         <v>45945</v>
       </c>
@@ -13730,21 +13796,21 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>MSI: SME resource and energy efficiency – industrial research</t>
+          <t>The Agentic AI Pioneers Prize</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2328/overview/79cb058a-71b3-459a-93c2-8c96ecf7f18a</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2316/overview/fa0eeab0-3021-4cbc-8975-5bd45a7d642a</t>
         </is>
       </c>
       <c r="D238" t="inlineStr">
         <is>
-          <t>2025-10-22 08:21</t>
+          <t>2025-10-21 08:20</t>
         </is>
       </c>
       <c r="E238" s="1" t="n">
-        <v>45952.34791666667</v>
+        <v>45951.34722222222</v>
       </c>
       <c r="F238" t="b">
         <v>1</v>
@@ -13757,19 +13823,15 @@
       <c r="J238" t="inlineStr"/>
       <c r="K238" t="inlineStr">
         <is>
-          <t>Wednesday 10 December 2025 11:00am</t>
+          <t>Wednesday 19 November 2025 11:00am</t>
         </is>
       </c>
       <c r="L238" s="1" t="n">
-        <v>46001.45833333334</v>
-      </c>
-      <c r="M238" t="inlineStr">
-        <is>
-          <t>£1.0 million</t>
-        </is>
-      </c>
+        <v>45980.45833333334</v>
+      </c>
+      <c r="M238" t="inlineStr"/>
       <c r="N238" s="1" t="n">
-        <v>45952</v>
+        <v>45945</v>
       </c>
     </row>
     <row r="239">
@@ -13780,12 +13842,12 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>MSI: SME resource and energy   efficiency – feasibility studies</t>
+          <t>MSI: SME resource and energy efficiency – industrial research</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2327/overview/bd7d1a37-69dc-4d09-8615-2bae4bcf3666</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2328/overview/79cb058a-71b3-459a-93c2-8c96ecf7f18a</t>
         </is>
       </c>
       <c r="D239" t="inlineStr">
@@ -13815,7 +13877,7 @@
       </c>
       <c r="M239" t="inlineStr">
         <is>
-          <t>£150,000</t>
+          <t>£1.0 million</t>
         </is>
       </c>
       <c r="N239" s="1" t="n">
@@ -13830,21 +13892,21 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>Full ADOPT Grant Round 4</t>
+          <t>MSI: SME resource and energy   efficiency – feasibility studies</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2298/overview/71fd7055-502d-4f85-9127-749156a80fe6</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2327/overview/bd7d1a37-69dc-4d09-8615-2bae4bcf3666</t>
         </is>
       </c>
       <c r="D240" t="inlineStr">
         <is>
-          <t>2025-10-23 08:19</t>
+          <t>2025-10-22 08:21</t>
         </is>
       </c>
       <c r="E240" s="1" t="n">
-        <v>45953.34652777778</v>
+        <v>45952.34791666667</v>
       </c>
       <c r="F240" t="b">
         <v>1</v>
@@ -13865,7 +13927,7 @@
       </c>
       <c r="M240" t="inlineStr">
         <is>
-          <t>£100,000</t>
+          <t>£150,000</t>
         </is>
       </c>
       <c r="N240" s="1" t="n">
@@ -13880,21 +13942,21 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>Innovate UK Innovation Loans Round 24</t>
+          <t>Full ADOPT Grant Round 4</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2322/overview/1b933876-5f58-4dec-85ab-68b8c2722211</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2298/overview/71fd7055-502d-4f85-9127-749156a80fe6</t>
         </is>
       </c>
       <c r="D241" t="inlineStr">
         <is>
-          <t>2025-10-24 08:19</t>
+          <t>2025-10-23 08:19</t>
         </is>
       </c>
       <c r="E241" s="1" t="n">
-        <v>45954.34652777778</v>
+        <v>45953.34652777778</v>
       </c>
       <c r="F241" t="b">
         <v>1</v>
@@ -13907,15 +13969,15 @@
       <c r="J241" t="inlineStr"/>
       <c r="K241" t="inlineStr">
         <is>
-          <t>Wednesday 7 January 2026 11:00am</t>
+          <t>Wednesday 10 December 2025 11:00am</t>
         </is>
       </c>
       <c r="L241" s="1" t="n">
-        <v>46029.45833333334</v>
+        <v>46001.45833333334</v>
       </c>
       <c r="M241" t="inlineStr">
         <is>
-          <t>£5.0 million</t>
+          <t>£100,000</t>
         </is>
       </c>
       <c r="N241" s="1" t="n">
@@ -13930,21 +13992,21 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>Knowledge Transfer Partnership (KTP): 2025 – 2026 Round 4</t>
+          <t>Innovate UK Innovation Loans Round 24</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2290/overview/8dd45f5c-3f38-4e38-b733-42b6cf601292</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2322/overview/1b933876-5f58-4dec-85ab-68b8c2722211</t>
         </is>
       </c>
       <c r="D242" t="inlineStr">
         <is>
-          <t>2025-10-25 08:16</t>
+          <t>2025-10-24 08:19</t>
         </is>
       </c>
       <c r="E242" s="1" t="n">
-        <v>45955.34444444445</v>
+        <v>45954.34652777778</v>
       </c>
       <c r="F242" t="b">
         <v>1</v>
@@ -13957,15 +14019,15 @@
       <c r="J242" t="inlineStr"/>
       <c r="K242" t="inlineStr">
         <is>
-          <t>Wednesday 26 November 2025 11:00am</t>
+          <t>Wednesday 7 January 2026 11:00am</t>
         </is>
       </c>
       <c r="L242" s="1" t="n">
-        <v>45987.45833333334</v>
+        <v>46029.45833333334</v>
       </c>
       <c r="M242" t="inlineStr">
         <is>
-          <t>£8,500</t>
+          <t>£5.0 million</t>
         </is>
       </c>
       <c r="N242" s="1" t="n">
@@ -13980,21 +14042,21 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>National Materials Innovation Programme: Feasibility Studies</t>
+          <t>Knowledge Transfer Partnership (KTP): 2025 – 2026 Round 4</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2326/overview/ca8aab61-a03b-431f-94a8-5c9b008495d5</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2290/overview/8dd45f5c-3f38-4e38-b733-42b6cf601292</t>
         </is>
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>2025-10-31 08:18</t>
+          <t>2025-10-25 08:16</t>
         </is>
       </c>
       <c r="E243" s="1" t="n">
-        <v>45961.34583333333</v>
+        <v>45955.34444444445</v>
       </c>
       <c r="F243" t="b">
         <v>1</v>
@@ -14007,19 +14069,19 @@
       <c r="J243" t="inlineStr"/>
       <c r="K243" t="inlineStr">
         <is>
-          <t>Wednesday 17 December 2025 11:00am</t>
+          <t>Wednesday 26 November 2025 11:00am</t>
         </is>
       </c>
       <c r="L243" s="1" t="n">
-        <v>46008.45833333334</v>
+        <v>45987.45833333334</v>
       </c>
       <c r="M243" t="inlineStr">
         <is>
-          <t>£100,000</t>
+          <t>£8,500</t>
         </is>
       </c>
       <c r="N243" s="1" t="n">
-        <v>45959</v>
+        <v>45952</v>
       </c>
     </row>
     <row r="244">
@@ -14030,21 +14092,21 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>UK-Canada Quantum Communications and Networking Demonstrator</t>
+          <t>National Materials Innovation Programme: Feasibility Studies</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2335/overview/64e26f1b-8564-4539-b3ca-1b15ebf4f94a</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2326/overview/ca8aab61-a03b-431f-94a8-5c9b008495d5</t>
         </is>
       </c>
       <c r="D244" t="inlineStr">
         <is>
-          <t>2025-11-04 08:20</t>
+          <t>2025-10-31 08:18</t>
         </is>
       </c>
       <c r="E244" s="1" t="n">
-        <v>45965.34722222222</v>
+        <v>45961.34583333333</v>
       </c>
       <c r="F244" t="b">
         <v>1</v>
@@ -14057,15 +14119,15 @@
       <c r="J244" t="inlineStr"/>
       <c r="K244" t="inlineStr">
         <is>
-          <t>Wednesday 26 November 2025 11:00am</t>
+          <t>Wednesday 17 December 2025 11:00am</t>
         </is>
       </c>
       <c r="L244" s="1" t="n">
-        <v>45987.45833333334</v>
+        <v>46008.45833333334</v>
       </c>
       <c r="M244" t="inlineStr">
         <is>
-          <t>£3.4 million</t>
+          <t>£100,000</t>
         </is>
       </c>
       <c r="N244" s="1" t="n">
@@ -14080,12 +14142,12 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>Increasing EV charging capacity on the strategic road network</t>
+          <t>UK-Canada Quantum Communications and Networking Demonstrator</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2304/overview/9ea6670e-83fd-43f9-972f-e0eff8fe77a8</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2335/overview/64e26f1b-8564-4539-b3ca-1b15ebf4f94a</t>
         </is>
       </c>
       <c r="D245" t="inlineStr">
@@ -14107,15 +14169,15 @@
       <c r="J245" t="inlineStr"/>
       <c r="K245" t="inlineStr">
         <is>
-          <t>Wednesday 25 March 2026 11:00am</t>
+          <t>Wednesday 26 November 2025 11:00am</t>
         </is>
       </c>
       <c r="L245" s="1" t="n">
-        <v>46106.45833333334</v>
+        <v>45987.45833333334</v>
       </c>
       <c r="M245" t="inlineStr">
         <is>
-          <t>£3.0 million</t>
+          <t>£3.4 million</t>
         </is>
       </c>
       <c r="N245" s="1" t="n">
@@ -14130,21 +14192,21 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>Biomedical Catalyst 2025: Industry led R&amp;D small projects</t>
+          <t>Increasing EV charging capacity on the strategic road network</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2333/overview/f5431c75-e2e1-48f4-bc8e-62d52121cb6f</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2304/overview/9ea6670e-83fd-43f9-972f-e0eff8fe77a8</t>
         </is>
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>2025-11-05 08:19</t>
+          <t>2025-11-04 08:20</t>
         </is>
       </c>
       <c r="E246" s="1" t="n">
-        <v>45966.34652777778</v>
+        <v>45965.34722222222</v>
       </c>
       <c r="F246" t="b">
         <v>1</v>
@@ -14157,19 +14219,19 @@
       <c r="J246" t="inlineStr"/>
       <c r="K246" t="inlineStr">
         <is>
-          <t>Wednesday 10 December 2025 11:00am</t>
+          <t>Wednesday 25 March 2026 11:00am</t>
         </is>
       </c>
       <c r="L246" s="1" t="n">
-        <v>46001.45833333334</v>
+        <v>46106.45833333334</v>
       </c>
       <c r="M246" t="inlineStr">
         <is>
-          <t>£1.0 million</t>
+          <t>£3.0 million</t>
         </is>
       </c>
       <c r="N246" s="1" t="n">
-        <v>45966</v>
+        <v>45959</v>
       </c>
     </row>
     <row r="247">
@@ -14180,12 +14242,12 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>Biomedical Catalyst 2025: Industry led R&amp;D large projects</t>
+          <t>Biomedical Catalyst 2025: Industry led R&amp;D small projects</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2332/overview/bf6bd8c3-e550-478d-b374-a3cb0fb4d3d3</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2333/overview/f5431c75-e2e1-48f4-bc8e-62d52121cb6f</t>
         </is>
       </c>
       <c r="D247" t="inlineStr">
@@ -14215,7 +14277,7 @@
       </c>
       <c r="M247" t="inlineStr">
         <is>
-          <t>£4.0 million</t>
+          <t>£1.0 million</t>
         </is>
       </c>
       <c r="N247" s="1" t="n">
@@ -14230,12 +14292,12 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>ATI Programme strategic batch EoI – November 2025</t>
+          <t>Biomedical Catalyst 2025: Industry led R&amp;D large projects</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2334/overview/4af06b80-2953-4cb3-8cc0-987ec5a2f322</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2332/overview/bf6bd8c3-e550-478d-b374-a3cb0fb4d3d3</t>
         </is>
       </c>
       <c r="D248" t="inlineStr">
@@ -14257,13 +14319,17 @@
       <c r="J248" t="inlineStr"/>
       <c r="K248" t="inlineStr">
         <is>
-          <t>Wednesday 19 November 2025 11:00am</t>
+          <t>Wednesday 10 December 2025 11:00am</t>
         </is>
       </c>
       <c r="L248" s="1" t="n">
-        <v>45980.45833333334</v>
-      </c>
-      <c r="M248" t="inlineStr"/>
+        <v>46001.45833333334</v>
+      </c>
+      <c r="M248" t="inlineStr">
+        <is>
+          <t>£4.0 million</t>
+        </is>
+      </c>
       <c r="N248" s="1" t="n">
         <v>45966</v>
       </c>
@@ -14276,21 +14342,21 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>DRIVE35 Scale-up: Feasibility Studies 2</t>
+          <t>ATI Programme strategic batch EoI – November 2025</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2341/overview/4b0efce9-75b8-4e84-97c0-fc6277396586</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2334/overview/4af06b80-2953-4cb3-8cc0-987ec5a2f322</t>
         </is>
       </c>
       <c r="D249" t="inlineStr">
         <is>
-          <t>2025-11-11 08:19</t>
+          <t>2025-11-05 08:19</t>
         </is>
       </c>
       <c r="E249" s="1" t="n">
-        <v>45972.34652777778</v>
+        <v>45966.34652777778</v>
       </c>
       <c r="F249" t="b">
         <v>1</v>
@@ -14303,17 +14369,13 @@
       <c r="J249" t="inlineStr"/>
       <c r="K249" t="inlineStr">
         <is>
-          <t>Wednesday 17 December 2025 11:00am</t>
+          <t>Wednesday 19 November 2025 11:00am</t>
         </is>
       </c>
       <c r="L249" s="1" t="n">
-        <v>46008.45833333334</v>
-      </c>
-      <c r="M249" t="inlineStr">
-        <is>
-          <t>£750,000</t>
-        </is>
-      </c>
+        <v>45980.45833333334</v>
+      </c>
+      <c r="M249" t="inlineStr"/>
       <c r="N249" s="1" t="n">
         <v>45966</v>
       </c>
@@ -14326,21 +14388,21 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>Women in Innovation Awards 2025/26</t>
+          <t>DRIVE35 Scale-up: Feasibility Studies 2</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2337/overview/3750b1cd-2080-4a1c-82c0-003fbaafdd2d</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2341/overview/4b0efce9-75b8-4e84-97c0-fc6277396586</t>
         </is>
       </c>
       <c r="D250" t="inlineStr">
         <is>
-          <t>2025-11-27 13:23</t>
+          <t>2025-11-11 08:19</t>
         </is>
       </c>
       <c r="E250" s="1" t="n">
-        <v>45988.55763888889</v>
+        <v>45972.34652777778</v>
       </c>
       <c r="F250" t="b">
         <v>1</v>
@@ -14353,19 +14415,19 @@
       <c r="J250" t="inlineStr"/>
       <c r="K250" t="inlineStr">
         <is>
-          <t>Wednesday 4 February 2026 11:00am</t>
+          <t>Wednesday 17 December 2025 11:00am</t>
         </is>
       </c>
       <c r="L250" s="1" t="n">
-        <v>46057.45833333334</v>
+        <v>46008.45833333334</v>
       </c>
       <c r="M250" t="inlineStr">
         <is>
-          <t>£75,000</t>
+          <t>£750,000</t>
         </is>
       </c>
       <c r="N250" s="1" t="n">
-        <v>45987</v>
+        <v>45966</v>
       </c>
     </row>
     <row r="251">
@@ -14376,21 +14438,21 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>Knowledge Transfer Partnership (KTP): 2025 – 2026 Round 5</t>
+          <t>Women in Innovation Awards 2025/26</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2354/overview/c7008321-f651-45c5-a409-c3215231fbb4</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2337/overview/3750b1cd-2080-4a1c-82c0-003fbaafdd2d</t>
         </is>
       </c>
       <c r="D251" t="inlineStr">
         <is>
-          <t>2025-12-02 08:22</t>
+          <t>2025-11-27 13:23</t>
         </is>
       </c>
       <c r="E251" s="1" t="n">
-        <v>45993.34861111111</v>
+        <v>45988.55763888889</v>
       </c>
       <c r="F251" t="b">
         <v>1</v>
@@ -14411,7 +14473,7 @@
       </c>
       <c r="M251" t="inlineStr">
         <is>
-          <t>£8,500</t>
+          <t>£75,000</t>
         </is>
       </c>
       <c r="N251" s="1" t="n">
@@ -14426,21 +14488,21 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>Innovate UK Growth Catalyst – Investor Partnerships Round 2</t>
+          <t>Knowledge Transfer Partnership (KTP): 2025 – 2026 Round 5</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2360/overview/37d8f6e1-5600-4e9e-bbfc-11bc320f8808</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2354/overview/c7008321-f651-45c5-a409-c3215231fbb4</t>
         </is>
       </c>
       <c r="D252" t="inlineStr">
         <is>
-          <t>2025-12-11 08:22</t>
+          <t>2025-12-02 08:22</t>
         </is>
       </c>
       <c r="E252" s="1" t="n">
-        <v>46002.34861111111</v>
+        <v>45993.34861111111</v>
       </c>
       <c r="F252" t="b">
         <v>1</v>
@@ -14453,19 +14515,19 @@
       <c r="J252" t="inlineStr"/>
       <c r="K252" t="inlineStr">
         <is>
-          <t>Tuesday 3 February 2026 11:00am</t>
+          <t>Wednesday 4 February 2026 11:00am</t>
         </is>
       </c>
       <c r="L252" s="1" t="n">
-        <v>46056.45833333334</v>
+        <v>46057.45833333334</v>
       </c>
       <c r="M252" t="inlineStr">
         <is>
-          <t>£2.0 million</t>
+          <t>£8,500</t>
         </is>
       </c>
       <c r="N252" s="1" t="n">
-        <v>46001</v>
+        <v>45987</v>
       </c>
     </row>
     <row r="253">
@@ -14476,21 +14538,21 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>Full ADOPT Grant: Round 5</t>
+          <t>Innovate UK Growth Catalyst – Investor Partnerships Round 2</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2358/overview/f93f32c2-dd04-474d-bc35-a8af1ecac1a9</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2360/overview/37d8f6e1-5600-4e9e-bbfc-11bc320f8808</t>
         </is>
       </c>
       <c r="D253" t="inlineStr">
         <is>
-          <t>2025-12-12 08:22</t>
+          <t>2025-12-11 08:22</t>
         </is>
       </c>
       <c r="E253" s="1" t="n">
-        <v>46003.34861111111</v>
+        <v>46002.34861111111</v>
       </c>
       <c r="F253" t="b">
         <v>1</v>
@@ -14503,15 +14565,15 @@
       <c r="J253" t="inlineStr"/>
       <c r="K253" t="inlineStr">
         <is>
-          <t>Wednesday 4 February 2026 11:00am</t>
+          <t>Tuesday 3 February 2026 11:00am</t>
         </is>
       </c>
       <c r="L253" s="1" t="n">
-        <v>46057.45833333334</v>
+        <v>46056.45833333334</v>
       </c>
       <c r="M253" t="inlineStr">
         <is>
-          <t>£100,000</t>
+          <t>£2.0 million</t>
         </is>
       </c>
       <c r="N253" s="1" t="n">
@@ -14526,21 +14588,21 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>ADOPT Facilitator Support Grant: Round 6</t>
+          <t>Full ADOPT Grant: Round 5</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2371/overview/471bfe91-9f9c-4086-a28a-15296f1957e2</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2358/overview/f93f32c2-dd04-474d-bc35-a8af1ecac1a9</t>
         </is>
       </c>
       <c r="D254" t="inlineStr">
         <is>
-          <t>2025-12-18 08:21</t>
+          <t>2025-12-12 08:22</t>
         </is>
       </c>
       <c r="E254" s="1" t="n">
-        <v>46009.34791666667</v>
+        <v>46003.34861111111</v>
       </c>
       <c r="F254" t="b">
         <v>1</v>
@@ -14553,19 +14615,19 @@
       <c r="J254" t="inlineStr"/>
       <c r="K254" t="inlineStr">
         <is>
-          <t>Wednesday 25 February 2026 11:00am</t>
+          <t>Wednesday 4 February 2026 11:00am</t>
         </is>
       </c>
       <c r="L254" s="1" t="n">
-        <v>46078.45833333334</v>
+        <v>46057.45833333334</v>
       </c>
       <c r="M254" t="inlineStr">
         <is>
-          <t>£2,500</t>
+          <t>£100,000</t>
         </is>
       </c>
       <c r="N254" s="1" t="n">
-        <v>46008</v>
+        <v>46001</v>
       </c>
     </row>
     <row r="255">
@@ -14576,12 +14638,12 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>Commercialising Knowledge Assets Fund (CKAF) Spring</t>
+          <t>ADOPT Facilitator Support Grant: Round 6</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2369/overview/abf7d399-81b9-4f33-b592-51825a288c37</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2371/overview/471bfe91-9f9c-4086-a28a-15296f1957e2</t>
         </is>
       </c>
       <c r="D255" t="inlineStr">
@@ -14603,15 +14665,15 @@
       <c r="J255" t="inlineStr"/>
       <c r="K255" t="inlineStr">
         <is>
-          <t>Thursday 7 May 2026 11:00am</t>
+          <t>Wednesday 25 February 2026 11:00am</t>
         </is>
       </c>
       <c r="L255" s="1" t="n">
-        <v>46149.45833333334</v>
+        <v>46078.45833333334</v>
       </c>
       <c r="M255" t="inlineStr">
         <is>
-          <t>£250,000</t>
+          <t>£2,500</t>
         </is>
       </c>
       <c r="N255" s="1" t="n">
@@ -14626,21 +14688,21 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>Energy catalyst round 11 – mid stage</t>
+          <t>Commercialising Knowledge Assets Fund (CKAF) Spring</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2363/overview/9f759af1-3732-4d15-995d-053e28025d22</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2369/overview/abf7d399-81b9-4f33-b592-51825a288c37</t>
         </is>
       </c>
       <c r="D256" t="inlineStr">
         <is>
-          <t>2026-01-06 08:22</t>
+          <t>2025-12-18 08:21</t>
         </is>
       </c>
       <c r="E256" s="1" t="n">
-        <v>46028.34861111111</v>
+        <v>46009.34791666667</v>
       </c>
       <c r="F256" t="b">
         <v>1</v>
@@ -14653,19 +14715,19 @@
       <c r="J256" t="inlineStr"/>
       <c r="K256" t="inlineStr">
         <is>
-          <t>Wednesday 25 March 2026 11:00am</t>
+          <t>Thursday 7 May 2026 11:00am</t>
         </is>
       </c>
       <c r="L256" s="1" t="n">
-        <v>46106.45833333334</v>
+        <v>46149.45833333334</v>
       </c>
       <c r="M256" t="inlineStr">
         <is>
-          <t>£1.5 million</t>
+          <t>£250,000</t>
         </is>
       </c>
       <c r="N256" s="1" t="n">
-        <v>46022</v>
+        <v>46008</v>
       </c>
     </row>
     <row r="257">
@@ -14676,12 +14738,12 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>Energy catalyst round 11 – late stage</t>
+          <t>Energy catalyst round 11 – mid stage</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2364/overview/b9d4dedf-d22a-41d1-9ca2-6c5a279519be</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2363/overview/9f759af1-3732-4d15-995d-053e28025d22</t>
         </is>
       </c>
       <c r="D257" t="inlineStr">
@@ -14711,7 +14773,7 @@
       </c>
       <c r="M257" t="inlineStr">
         <is>
-          <t>£5.0 million</t>
+          <t>£1.5 million</t>
         </is>
       </c>
       <c r="N257" s="1" t="n">
@@ -14726,12 +14788,12 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>Energy catalyst round 11 – early stage</t>
+          <t>Energy catalyst round 11 – late stage</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2362/overview/640b2f4e-8571-4aef-9e2a-67e35db3db77</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2364/overview/b9d4dedf-d22a-41d1-9ca2-6c5a279519be</t>
         </is>
       </c>
       <c r="D258" t="inlineStr">
@@ -14761,7 +14823,7 @@
       </c>
       <c r="M258" t="inlineStr">
         <is>
-          <t>£300,000</t>
+          <t>£5.0 million</t>
         </is>
       </c>
       <c r="N258" s="1" t="n">
@@ -14776,12 +14838,12 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>DRIVE35 Innovation Fund: Demonstrate 2</t>
+          <t>Energy catalyst round 11 – early stage</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2351/overview/349c38f5-5ed2-4cf4-a324-bda2d6cd1e67</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2362/overview/640b2f4e-8571-4aef-9e2a-67e35db3db77</t>
         </is>
       </c>
       <c r="D259" t="inlineStr">
@@ -14803,15 +14865,15 @@
       <c r="J259" t="inlineStr"/>
       <c r="K259" t="inlineStr">
         <is>
-          <t>Wednesday 11 March 2026 11:00am</t>
+          <t>Wednesday 25 March 2026 11:00am</t>
         </is>
       </c>
       <c r="L259" s="1" t="n">
-        <v>46092.45833333334</v>
+        <v>46106.45833333334</v>
       </c>
       <c r="M259" t="inlineStr">
         <is>
-          <t>£1.5 million</t>
+          <t>£300,000</t>
         </is>
       </c>
       <c r="N259" s="1" t="n">
@@ -14826,12 +14888,12 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>DRIVE35 Innovation Fund: Collaborate 2</t>
+          <t>DRIVE35 Innovation Fund: Demonstrate 2</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2350/overview/dbd41be3-14ea-4c83-8774-eb28a8703d57</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2351/overview/349c38f5-5ed2-4cf4-a324-bda2d6cd1e67</t>
         </is>
       </c>
       <c r="D260" t="inlineStr">
@@ -14853,15 +14915,15 @@
       <c r="J260" t="inlineStr"/>
       <c r="K260" t="inlineStr">
         <is>
-          <t>Wednesday 18 March 2026 11:00am</t>
+          <t>Wednesday 11 March 2026 11:00am</t>
         </is>
       </c>
       <c r="L260" s="1" t="n">
-        <v>46099.45833333334</v>
+        <v>46092.45833333334</v>
       </c>
       <c r="M260" t="inlineStr">
         <is>
-          <t>£25.0 million</t>
+          <t>£1.5 million</t>
         </is>
       </c>
       <c r="N260" s="1" t="n">
@@ -14876,21 +14938,21 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>Innovate UK Innovation Loans Round 25</t>
+          <t>DRIVE35 Innovation Fund: Collaborate 2</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2373/overview/609dc5dd-d3e8-4f51-af3a-3eb1b3314710</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2350/overview/dbd41be3-14ea-4c83-8774-eb28a8703d57</t>
         </is>
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>2026-01-08 08:22</t>
+          <t>2026-01-06 08:22</t>
         </is>
       </c>
       <c r="E261" s="1" t="n">
-        <v>46030.34861111111</v>
+        <v>46028.34861111111</v>
       </c>
       <c r="F261" t="b">
         <v>1</v>
@@ -14903,19 +14965,19 @@
       <c r="J261" t="inlineStr"/>
       <c r="K261" t="inlineStr">
         <is>
-          <t>Wednesday 4 March 2026 11:00am</t>
+          <t>Wednesday 18 March 2026 11:00am</t>
         </is>
       </c>
       <c r="L261" s="1" t="n">
-        <v>46085.45833333334</v>
+        <v>46099.45833333334</v>
       </c>
       <c r="M261" t="inlineStr">
         <is>
-          <t>£5.0 million</t>
+          <t>£25.0 million</t>
         </is>
       </c>
       <c r="N261" s="1" t="n">
-        <v>46029</v>
+        <v>46022</v>
       </c>
     </row>
     <row r="262">
@@ -14926,21 +14988,21 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>Cyber Security Academic Startup Accelerator Programme Y10 Phase 1</t>
+          <t>Innovate UK Innovation Loans Round 25</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2376/overview/1b9b9265-ca4b-4f8c-a0c2-577cb8713642</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2373/overview/609dc5dd-d3e8-4f51-af3a-3eb1b3314710</t>
         </is>
       </c>
       <c r="D262" t="inlineStr">
         <is>
-          <t>2026-01-15 08:23</t>
+          <t>2026-01-08 08:22</t>
         </is>
       </c>
       <c r="E262" s="1" t="n">
-        <v>46037.34930555556</v>
+        <v>46030.34861111111</v>
       </c>
       <c r="F262" t="b">
         <v>1</v>
@@ -14953,19 +15015,19 @@
       <c r="J262" t="inlineStr"/>
       <c r="K262" t="inlineStr">
         <is>
-          <t>Wednesday 11 February 2026 11:00am</t>
+          <t>Wednesday 4 March 2026 11:00am</t>
         </is>
       </c>
       <c r="L262" s="1" t="n">
-        <v>46064.45833333334</v>
+        <v>46085.45833333334</v>
       </c>
       <c r="M262" t="inlineStr">
         <is>
-          <t>£32,000</t>
+          <t>£5.0 million</t>
         </is>
       </c>
       <c r="N262" s="1" t="n">
-        <v>46036</v>
+        <v>46029</v>
       </c>
     </row>
     <row r="263">
@@ -14976,21 +15038,21 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>Ofgem Strategic Innovation Fund Round 5 Discovery C5</t>
+          <t>Cyber Security Academic Startup Accelerator Programme Y10 Phase 1</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2346/overview/e172ee7c-3050-4d47-bf11-235cfe76c1e1</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2376/overview/1b9b9265-ca4b-4f8c-a0c2-577cb8713642</t>
         </is>
       </c>
       <c r="D263" t="inlineStr">
         <is>
-          <t>2026-01-20 08:24</t>
+          <t>2026-01-15 08:23</t>
         </is>
       </c>
       <c r="E263" s="1" t="n">
-        <v>46042.35</v>
+        <v>46037.34930555556</v>
       </c>
       <c r="F263" t="b">
         <v>1</v>
@@ -15003,15 +15065,15 @@
       <c r="J263" t="inlineStr"/>
       <c r="K263" t="inlineStr">
         <is>
-          <t>Wednesday 25 February 2026 11:00am</t>
+          <t>Wednesday 11 February 2026 11:00am</t>
         </is>
       </c>
       <c r="L263" s="1" t="n">
-        <v>46078.45833333334</v>
+        <v>46064.45833333334</v>
       </c>
       <c r="M263" t="inlineStr">
         <is>
-          <t>£150,000</t>
+          <t>£32,000</t>
         </is>
       </c>
       <c r="N263" s="1" t="n">
@@ -15026,21 +15088,21 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>Advanced manufacturing supply chain innovation FS</t>
+          <t>Ofgem Strategic Innovation Fund Round 5 Discovery C5</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2384/overview/2ad8ce21-d3f6-48bf-b55a-5af2a892a1e0</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2346/overview/e172ee7c-3050-4d47-bf11-235cfe76c1e1</t>
         </is>
       </c>
       <c r="D264" t="inlineStr">
         <is>
-          <t>2026-01-26 12:10</t>
+          <t>2026-01-20 08:24</t>
         </is>
       </c>
       <c r="E264" s="1" t="n">
-        <v>46048.50694444445</v>
+        <v>46042.35</v>
       </c>
       <c r="F264" t="b">
         <v>1</v>
@@ -15053,19 +15115,19 @@
       <c r="J264" t="inlineStr"/>
       <c r="K264" t="inlineStr">
         <is>
-          <t>Wednesday 11 March 2026 11:00am</t>
+          <t>Wednesday 25 February 2026 11:00am</t>
         </is>
       </c>
       <c r="L264" s="1" t="n">
-        <v>46092.45833333334</v>
+        <v>46078.45833333334</v>
       </c>
       <c r="M264" t="inlineStr">
         <is>
-          <t>£100,000</t>
+          <t>£150,000</t>
         </is>
       </c>
       <c r="N264" s="1" t="n">
-        <v>46043</v>
+        <v>46036</v>
       </c>
     </row>
     <row r="265">
@@ -15076,21 +15138,21 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>TechLocal: Connecting Local Talent to Local Tech Jobs</t>
+          <t>Advanced manufacturing supply chain innovation FS</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2378/overview/ae120ce2-7b72-4cf2-8dde-f78b02d5996d</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2384/overview/2ad8ce21-d3f6-48bf-b55a-5af2a892a1e0</t>
         </is>
       </c>
       <c r="D265" t="inlineStr">
         <is>
-          <t>2026-01-28 10:24</t>
+          <t>2026-01-26 12:10</t>
         </is>
       </c>
       <c r="E265" s="1" t="n">
-        <v>46050.43333333333</v>
+        <v>46048.50694444445</v>
       </c>
       <c r="F265" t="b">
         <v>1</v>
@@ -15103,19 +15165,19 @@
       <c r="J265" t="inlineStr"/>
       <c r="K265" t="inlineStr">
         <is>
-          <t>Wednesday 18 March 2026 11:00am</t>
+          <t>Wednesday 11 March 2026 11:00am</t>
         </is>
       </c>
       <c r="L265" s="1" t="n">
-        <v>46099.45833333334</v>
+        <v>46092.45833333334</v>
       </c>
       <c r="M265" t="inlineStr">
         <is>
-          <t>£225,000</t>
+          <t>£100,000</t>
         </is>
       </c>
       <c r="N265" s="1" t="n">
-        <v>46050</v>
+        <v>46043</v>
       </c>
     </row>
     <row r="266">
@@ -15126,12 +15188,12 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>TechLocal AI Professional Degree and Traineeship Accelerator</t>
+          <t>TechLocal: Connecting Local Talent to Local Tech Jobs</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2375/overview/6431359e-eb5c-4f76-b49d-299948107fbd</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2378/overview/ae120ce2-7b72-4cf2-8dde-f78b02d5996d</t>
         </is>
       </c>
       <c r="D266" t="inlineStr">
@@ -15161,7 +15223,7 @@
       </c>
       <c r="M266" t="inlineStr">
         <is>
-          <t>£300,000</t>
+          <t>£225,000</t>
         </is>
       </c>
       <c r="N266" s="1" t="n">
@@ -15176,21 +15238,21 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>Robotics Adoption Programme skills development</t>
+          <t>TechLocal AI Professional Degree and Traineeship Accelerator</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2387/overview/daca31c2-8395-4bc2-a5da-55eb1e432fa4</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2375/overview/6431359e-eb5c-4f76-b49d-299948107fbd</t>
         </is>
       </c>
       <c r="D267" t="inlineStr">
         <is>
-          <t>2026-02-02 10:39</t>
+          <t>2026-01-28 10:24</t>
         </is>
       </c>
       <c r="E267" s="1" t="n">
-        <v>46055.44375</v>
+        <v>46050.43333333333</v>
       </c>
       <c r="F267" t="b">
         <v>1</v>
@@ -15203,15 +15265,15 @@
       <c r="J267" t="inlineStr"/>
       <c r="K267" t="inlineStr">
         <is>
-          <t>Wednesday 25 March 2026 11:00am</t>
+          <t>Wednesday 18 March 2026 11:00am</t>
         </is>
       </c>
       <c r="L267" s="1" t="n">
-        <v>46106.45833333334</v>
+        <v>46099.45833333334</v>
       </c>
       <c r="M267" t="inlineStr">
         <is>
-          <t>£500,000</t>
+          <t>£300,000</t>
         </is>
       </c>
       <c r="N267" s="1" t="n">
@@ -15226,21 +15288,21 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>Knowledge Transfer Partnership (KTP): 2026 – 2027 Round 1</t>
+          <t>Robotics Adoption Programme skills development</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2380/overview/3e170dd3-4458-4c7e-a096-e0ea50b88040</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2387/overview/daca31c2-8395-4bc2-a5da-55eb1e432fa4</t>
         </is>
       </c>
       <c r="D268" t="inlineStr">
         <is>
-          <t>2026-02-03 10:35</t>
+          <t>2026-02-02 10:39</t>
         </is>
       </c>
       <c r="E268" s="1" t="n">
-        <v>46056.44097222222</v>
+        <v>46055.44375</v>
       </c>
       <c r="F268" t="b">
         <v>1</v>
@@ -15253,15 +15315,15 @@
       <c r="J268" t="inlineStr"/>
       <c r="K268" t="inlineStr">
         <is>
-          <t>Wednesday 1 April 2026 11:00am</t>
+          <t>Wednesday 25 March 2026 11:00am</t>
         </is>
       </c>
       <c r="L268" s="1" t="n">
-        <v>46113.45833333334</v>
+        <v>46106.45833333334</v>
       </c>
       <c r="M268" t="inlineStr">
         <is>
-          <t>£8,500</t>
+          <t>£500,000</t>
         </is>
       </c>
       <c r="N268" s="1" t="n">
@@ -15276,12 +15338,12 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>Biomedical Catalyst Accelerator Provider Pool EoI: late stage</t>
+          <t>Knowledge Transfer Partnership (KTP): 2026 – 2027 Round 1</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2389/overview/a7f7d874-8b6b-45d6-b1e1-1e88e11a1ea5</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2380/overview/3e170dd3-4458-4c7e-a096-e0ea50b88040</t>
         </is>
       </c>
       <c r="D269" t="inlineStr">
@@ -15303,13 +15365,17 @@
       <c r="J269" t="inlineStr"/>
       <c r="K269" t="inlineStr">
         <is>
-          <t>Wednesday 4 March 2026 11:00am</t>
+          <t>Wednesday 1 April 2026 11:00am</t>
         </is>
       </c>
       <c r="L269" s="1" t="n">
-        <v>46085.45833333334</v>
-      </c>
-      <c r="M269" t="inlineStr"/>
+        <v>46113.45833333334</v>
+      </c>
+      <c r="M269" t="inlineStr">
+        <is>
+          <t>£8,500</t>
+        </is>
+      </c>
       <c r="N269" s="1" t="n">
         <v>46050</v>
       </c>
@@ -15322,12 +15388,12 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>Biomedical Catalyst Accelerator Provider Pool EoI: early stage</t>
+          <t>Biomedical Catalyst Accelerator Provider Pool EoI: late stage</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2388/overview/08b8ab63-085d-4d79-ae83-e8c1698cb327</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2389/overview/a7f7d874-8b6b-45d6-b1e1-1e88e11a1ea5</t>
         </is>
       </c>
       <c r="D270" t="inlineStr">
@@ -15368,21 +15434,21 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>Full ADOPT Grant: Round 6</t>
+          <t>Biomedical Catalyst Accelerator Provider Pool EoI: early stage</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2385/overview/2343c344-807d-41a1-9551-05ac5420ba11</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2388/overview/08b8ab63-085d-4d79-ae83-e8c1698cb327</t>
         </is>
       </c>
       <c r="D271" t="inlineStr">
         <is>
-          <t>2026-02-09 10:53</t>
+          <t>2026-02-03 10:35</t>
         </is>
       </c>
       <c r="E271" s="1" t="n">
-        <v>46062.45347222222</v>
+        <v>46056.44097222222</v>
       </c>
       <c r="F271" t="b">
         <v>1</v>
@@ -15395,19 +15461,15 @@
       <c r="J271" t="inlineStr"/>
       <c r="K271" t="inlineStr">
         <is>
-          <t>Wednesday 8 April 2026 11:00am</t>
+          <t>Wednesday 4 March 2026 11:00am</t>
         </is>
       </c>
       <c r="L271" s="1" t="n">
-        <v>46120.45833333334</v>
-      </c>
-      <c r="M271" t="inlineStr">
-        <is>
-          <t>£100,000</t>
-        </is>
-      </c>
+        <v>46085.45833333334</v>
+      </c>
+      <c r="M271" t="inlineStr"/>
       <c r="N271" s="1" t="n">
-        <v>46057</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="272">
@@ -15418,21 +15480,21 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>Zero Emission Flight Demonstrator Round 1</t>
+          <t>Full ADOPT Grant: Round 6</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2397/overview/752074ec-5f01-46d8-863f-596300a11651</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2385/overview/2343c344-807d-41a1-9551-05ac5420ba11</t>
         </is>
       </c>
       <c r="D272" t="inlineStr">
         <is>
-          <t>2026-02-12 10:40</t>
+          <t>2026-02-09 10:53</t>
         </is>
       </c>
       <c r="E272" s="1" t="n">
-        <v>46065.44444444445</v>
+        <v>46062.45347222222</v>
       </c>
       <c r="F272" t="b">
         <v>1</v>
@@ -15445,19 +15507,19 @@
       <c r="J272" t="inlineStr"/>
       <c r="K272" t="inlineStr">
         <is>
-          <t>Wednesday 1 April 2026 11:00am</t>
+          <t>Wednesday 8 April 2026 11:00am</t>
         </is>
       </c>
       <c r="L272" s="1" t="n">
-        <v>46113.45833333334</v>
+        <v>46120.45833333334</v>
       </c>
       <c r="M272" t="inlineStr">
         <is>
-          <t>£5.0 million</t>
+          <t>£100,000</t>
         </is>
       </c>
       <c r="N272" s="1" t="n">
-        <v>46064</v>
+        <v>46057</v>
       </c>
     </row>
     <row r="273">
@@ -15468,12 +15530,12 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>Contracts for Innovation in drug and alcohol addiction healthcare</t>
+          <t>Zero Emission Flight Demonstrator Round 1</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2395/overview/3d49fbc4-6e09-4dd8-9ac8-8e5f88facd8d</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2397/overview/752074ec-5f01-46d8-863f-596300a11651</t>
         </is>
       </c>
       <c r="D273" t="inlineStr">
@@ -15495,15 +15557,15 @@
       <c r="J273" t="inlineStr"/>
       <c r="K273" t="inlineStr">
         <is>
-          <t>Wednesday 6 May 2026 11:00am</t>
+          <t>Wednesday 1 April 2026 11:00am</t>
         </is>
       </c>
       <c r="L273" s="1" t="n">
-        <v>46148.45833333334</v>
+        <v>46113.45833333334</v>
       </c>
       <c r="M273" t="inlineStr">
         <is>
-          <t>£1.5 million</t>
+          <t>£5.0 million</t>
         </is>
       </c>
       <c r="N273" s="1" t="n">
@@ -15518,12 +15580,12 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>Advancing innovation in drug and alcohol addiction healthcare</t>
+          <t>Contracts for Innovation in drug and alcohol addiction healthcare</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2394/overview/33b56af8-353f-46ac-bb66-a0928731c0fc</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2395/overview/3d49fbc4-6e09-4dd8-9ac8-8e5f88facd8d</t>
         </is>
       </c>
       <c r="D274" t="inlineStr">
@@ -15553,7 +15615,7 @@
       </c>
       <c r="M274" t="inlineStr">
         <is>
-          <t>£10.0 million</t>
+          <t>£1.5 million</t>
         </is>
       </c>
       <c r="N274" s="1" t="n">
@@ -15568,21 +15630,21 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>UK-Germany Collaborative Innovation for Quantum Technologies 2026</t>
+          <t>Advancing innovation in drug and alcohol addiction healthcare</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2392/overview/b8b93732-6326-4aed-9af3-334e4cc5ecc0</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2394/overview/33b56af8-353f-46ac-bb66-a0928731c0fc</t>
         </is>
       </c>
       <c r="D275" t="inlineStr">
         <is>
-          <t>2026-02-13 10:35</t>
+          <t>2026-02-12 10:40</t>
         </is>
       </c>
       <c r="E275" s="1" t="n">
-        <v>46066.44097222222</v>
+        <v>46065.44444444445</v>
       </c>
       <c r="F275" t="b">
         <v>1</v>
@@ -15595,15 +15657,15 @@
       <c r="J275" t="inlineStr"/>
       <c r="K275" t="inlineStr">
         <is>
-          <t>Wednesday 15 April 2026 11:00am</t>
+          <t>Wednesday 6 May 2026 11:00am</t>
         </is>
       </c>
       <c r="L275" s="1" t="n">
-        <v>46127.45833333334</v>
+        <v>46148.45833333334</v>
       </c>
       <c r="M275" t="inlineStr">
         <is>
-          <t>£1.0 million</t>
+          <t>£10.0 million</t>
         </is>
       </c>
       <c r="N275" s="1" t="n">
@@ -15618,21 +15680,21 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>Contracts for Innovation: industrial human relevant drug models</t>
+          <t>UK-Germany Collaborative Innovation for Quantum Technologies 2026</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2396/overview/d55398bb-ff62-43b9-9ee1-bf3fa4b95c5c</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2392/overview/b8b93732-6326-4aed-9af3-334e4cc5ecc0</t>
         </is>
       </c>
       <c r="D276" t="inlineStr">
         <is>
-          <t>2026-02-17 10:40</t>
+          <t>2026-02-13 10:35</t>
         </is>
       </c>
       <c r="E276" s="1" t="n">
-        <v>46070.44444444445</v>
+        <v>46066.44097222222</v>
       </c>
       <c r="F276" t="b">
         <v>1</v>
@@ -15653,7 +15715,7 @@
       </c>
       <c r="M276" t="inlineStr">
         <is>
-          <t>£200,000</t>
+          <t>£1.0 million</t>
         </is>
       </c>
       <c r="N276" s="1" t="n">
@@ -15668,21 +15730,21 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>Semiconductors and components for smart electronic platforms</t>
+          <t>Contracts for Innovation: industrial human relevant drug models</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2403/overview/4b54c133-c9b2-4572-9cca-2a7a4f69e5b8</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2396/overview/d55398bb-ff62-43b9-9ee1-bf3fa4b95c5c</t>
         </is>
       </c>
       <c r="D277" t="inlineStr">
         <is>
-          <t>2026-02-20 10:32</t>
+          <t>2026-02-17 10:40</t>
         </is>
       </c>
       <c r="E277" s="1" t="n">
-        <v>46073.43888888889</v>
+        <v>46070.44444444445</v>
       </c>
       <c r="F277" t="b">
         <v>1</v>
@@ -15695,19 +15757,19 @@
       <c r="J277" t="inlineStr"/>
       <c r="K277" t="inlineStr">
         <is>
-          <t>Wednesday 1 April 2026 11:00am</t>
+          <t>Wednesday 15 April 2026 11:00am</t>
         </is>
       </c>
       <c r="L277" s="1" t="n">
-        <v>46113.45833333334</v>
+        <v>46127.45833333334</v>
       </c>
       <c r="M277" t="inlineStr">
         <is>
-          <t>£2.0 million</t>
+          <t>£200,000</t>
         </is>
       </c>
       <c r="N277" s="1" t="n">
-        <v>46071</v>
+        <v>46064</v>
       </c>
     </row>
     <row r="278">
@@ -15718,21 +15780,21 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>Robotics Adoption Hubs</t>
+          <t>Semiconductors and components for smart electronic platforms</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2408/overview/ad7d7d36-af60-48be-91b0-f3208cf7c1d4</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2403/overview/4b54c133-c9b2-4572-9cca-2a7a4f69e5b8</t>
         </is>
       </c>
       <c r="D278" t="inlineStr">
         <is>
-          <t>2026-02-24 10:43</t>
+          <t>2026-02-20 10:32</t>
         </is>
       </c>
       <c r="E278" s="1" t="n">
-        <v>46077.44652777778</v>
+        <v>46073.43888888889</v>
       </c>
       <c r="F278" t="b">
         <v>1</v>
@@ -15745,15 +15807,15 @@
       <c r="J278" t="inlineStr"/>
       <c r="K278" t="inlineStr">
         <is>
-          <t>Wednesday 15 April 2026 11:00am</t>
+          <t>Wednesday 1 April 2026 11:00am</t>
         </is>
       </c>
       <c r="L278" s="1" t="n">
-        <v>46127.45833333334</v>
+        <v>46113.45833333334</v>
       </c>
       <c r="M278" t="inlineStr">
         <is>
-          <t>£7.5 million</t>
+          <t>£2.0 million</t>
         </is>
       </c>
       <c r="N278" s="1" t="n">
@@ -15768,12 +15830,12 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>Robotics Adoption Central Convening Body</t>
+          <t>Robotics Adoption Hubs</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2409/overview/c7e5dd6a-9f34-4614-b548-214b76190c14</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2408/overview/ad7d7d36-af60-48be-91b0-f3208cf7c1d4</t>
         </is>
       </c>
       <c r="D279" t="inlineStr">
@@ -15803,7 +15865,7 @@
       </c>
       <c r="M279" t="inlineStr">
         <is>
-          <t>£2.0 million</t>
+          <t>£7.5 million</t>
         </is>
       </c>
       <c r="N279" s="1" t="n">
@@ -15818,21 +15880,21 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>ADOPT Facilitator Support Grant: Round 7</t>
+          <t>Robotics Adoption Central Convening Body</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2404/overview/99693fa4-0f17-4de8-b812-34f2be37a4d0</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2409/overview/c7e5dd6a-9f34-4614-b548-214b76190c14</t>
         </is>
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>2026-02-26 10:40</t>
+          <t>2026-02-24 10:43</t>
         </is>
       </c>
       <c r="E280" s="1" t="n">
-        <v>46079.44444444445</v>
+        <v>46077.44652777778</v>
       </c>
       <c r="F280" t="b">
         <v>1</v>
@@ -15845,19 +15907,19 @@
       <c r="J280" t="inlineStr"/>
       <c r="K280" t="inlineStr">
         <is>
-          <t>Wednesday 8 April 2026 11:00am</t>
+          <t>Wednesday 15 April 2026 11:00am</t>
         </is>
       </c>
       <c r="L280" s="1" t="n">
-        <v>46120.45833333334</v>
+        <v>46127.45833333334</v>
       </c>
       <c r="M280" t="inlineStr">
         <is>
-          <t>£2,500</t>
+          <t>£2.0 million</t>
         </is>
       </c>
       <c r="N280" s="1" t="n">
-        <v>46078</v>
+        <v>46071</v>
       </c>
     </row>
     <row r="281">
@@ -15868,21 +15930,21 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>SNPN 5G Assured Integration (CR&amp;D)</t>
+          <t>ADOPT Facilitator Support Grant: Round 7</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2400/overview/cbbc48e2-d78e-42cd-b570-330f702ba82f</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2404/overview/99693fa4-0f17-4de8-b812-34f2be37a4d0</t>
         </is>
       </c>
       <c r="D281" t="inlineStr">
         <is>
-          <t>2026-03-03 10:34</t>
+          <t>2026-02-26 10:40</t>
         </is>
       </c>
       <c r="E281" s="1" t="n">
-        <v>46084.44027777778</v>
+        <v>46079.44444444445</v>
       </c>
       <c r="F281" t="b">
         <v>1</v>
@@ -15895,15 +15957,15 @@
       <c r="J281" t="inlineStr"/>
       <c r="K281" t="inlineStr">
         <is>
-          <t>Wednesday 1 April 2026 11:00am</t>
+          <t>Wednesday 8 April 2026 11:00am</t>
         </is>
       </c>
       <c r="L281" s="1" t="n">
-        <v>46113.45833333334</v>
+        <v>46120.45833333334</v>
       </c>
       <c r="M281" t="inlineStr">
         <is>
-          <t>£4.0 million</t>
+          <t>£2,500</t>
         </is>
       </c>
       <c r="N281" s="1" t="n">
@@ -15918,21 +15980,21 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>Clean Maritime Demonstration Competition 7: Pre-deployment trials</t>
+          <t>SNPN 5G Assured Integration (CR&amp;D)</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2415/overview/fa34afe8-b2e7-4cda-b77b-cf952d26a27a</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2400/overview/cbbc48e2-d78e-42cd-b570-330f702ba82f</t>
         </is>
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>2026-03-11 10:34</t>
+          <t>2026-03-03 10:34</t>
         </is>
       </c>
       <c r="E282" s="1" t="n">
-        <v>46092.44027777778</v>
+        <v>46084.44027777778</v>
       </c>
       <c r="F282" t="b">
         <v>1</v>
@@ -15945,19 +16007,19 @@
       <c r="J282" t="inlineStr"/>
       <c r="K282" t="inlineStr">
         <is>
-          <t>Wednesday 15 July 2026 11:00am</t>
+          <t>Wednesday 1 April 2026 11:00am</t>
         </is>
       </c>
       <c r="L282" s="1" t="n">
-        <v>46218.45833333334</v>
+        <v>46113.45833333334</v>
       </c>
       <c r="M282" t="inlineStr">
         <is>
-          <t>£6.0 million</t>
+          <t>£4.0 million</t>
         </is>
       </c>
       <c r="N282" s="1" t="n">
-        <v>46092</v>
+        <v>46078</v>
       </c>
     </row>
     <row r="283">
@@ -15968,12 +16030,12 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>Clean Maritime Demonstration Competition 7: Feasibility studies</t>
+          <t>Clean Maritime Demonstration Competition 7: Pre-deployment trials</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2416/overview/f49610a2-5e82-4898-b357-10f80154a2b8</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2415/overview/fa34afe8-b2e7-4cda-b77b-cf952d26a27a</t>
         </is>
       </c>
       <c r="D283" t="inlineStr">
@@ -16003,7 +16065,7 @@
       </c>
       <c r="M283" t="inlineStr">
         <is>
-          <t>£1.0 million</t>
+          <t>£6.0 million</t>
         </is>
       </c>
       <c r="N283" s="1" t="n">
@@ -16018,12 +16080,12 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>Clean Maritime Demonstration Competition 7: Deployment trials</t>
+          <t>Clean Maritime Demonstration Competition 7: Feasibility studies</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2414/overview/3409b968-a2b7-44e7-83a7-c2d3e8ad8f8e</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2416/overview/f49610a2-5e82-4898-b357-10f80154a2b8</t>
         </is>
       </c>
       <c r="D284" t="inlineStr">
@@ -16053,10 +16115,60 @@
       </c>
       <c r="M284" t="inlineStr">
         <is>
+          <t>£1.0 million</t>
+        </is>
+      </c>
+      <c r="N284" s="1" t="n">
+        <v>46092</v>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>Innovate Funding Service</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>Clean Maritime Demonstration Competition 7: Deployment trials</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2414/overview/3409b968-a2b7-44e7-83a7-c2d3e8ad8f8e</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>2026-03-11 10:34</t>
+        </is>
+      </c>
+      <c r="E285" s="1" t="n">
+        <v>46092.44027777778</v>
+      </c>
+      <c r="F285" t="b">
+        <v>1</v>
+      </c>
+      <c r="G285" t="inlineStr"/>
+      <c r="H285" t="b">
+        <v>0</v>
+      </c>
+      <c r="I285" t="inlineStr"/>
+      <c r="J285" t="inlineStr"/>
+      <c r="K285" t="inlineStr">
+        <is>
+          <t>Wednesday 15 July 2026 11:00am</t>
+        </is>
+      </c>
+      <c r="L285" s="1" t="n">
+        <v>46218.45833333334</v>
+      </c>
+      <c r="M285" t="inlineStr">
+        <is>
           <t>£15.0 million</t>
         </is>
       </c>
-      <c r="N284" s="1" t="n">
+      <c r="N285" s="1" t="n">
         <v>46092</v>
       </c>
     </row>
@@ -16098,10 +16210,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C2" t="n">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="3">
@@ -16124,10 +16236,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="C4" t="n">
-        <v>283</v>
+        <v>284</v>
       </c>
     </row>
     <row r="5">

</xml_diff>